<commit_message>
Loki's cost (80g, read in game — the map carries none) + new cost_source column
</commit_message>
<xml_diff>
--- a/skibi-data.xlsx
+++ b/skibi-data.xlsx
@@ -30,23 +30,23 @@
     <sheet name="waves" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'arcane'!$A$1:$AU$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'arcane'!$A$1:$AV$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'armour_matrix'!$A$1:$F$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'bosses'!$A$1:$O$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'caster_dps'!$A$1:$L$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'game_modes'!$A$1:$I$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'hero_ranking'!$A$1:$J$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'heroes'!$A$1:$H$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'military'!$A$1:$AX$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'military'!$A$1:$AY$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'minigame_items'!$A$1:$D$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'minigame_readings'!$A$1:$G$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'minigames'!$A$1:$I$80</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'other_towers'!$A$1:$AV$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'ranger'!$A$1:$AU$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'royal_family'!$A$1:$BA$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'scarlet_knight'!$A$1:$AU$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'specialist'!$A$1:$AY$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'tempest'!$A$1:$BA$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'other_towers'!$A$1:$AW$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'ranger'!$A$1:$AV$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'royal_family'!$A$1:$BB$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'scarlet_knight'!$A$1:$AV$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'specialist'!$A$1:$AZ$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'tempest'!$A$1:$BB$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'tower_traits'!$A$1:$I$113</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'wave_modifiers'!$A$1:$D$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'wave_traits'!$A$1:$K$51</definedName>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU18"/>
+  <dimension ref="A1:AV18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -513,6 +513,7 @@
     <col width="15" customWidth="1" min="45" max="45"/>
     <col width="22" customWidth="1" min="46" max="46"/>
     <col width="48" customWidth="1" min="47" max="47"/>
+    <col width="13" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -751,6 +752,11 @@
           <t>dps_source</t>
         </is>
       </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>cost_source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -828,6 +834,11 @@
           <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
         </is>
       </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -907,6 +918,11 @@
           <t>caster: Arctic Blast (sustained, mana-limited)</t>
         </is>
       </c>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -984,6 +1000,11 @@
           <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
         </is>
       </c>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1063,6 +1084,11 @@
           <t>caster: Scald (sustained, mana-limited)</t>
         </is>
       </c>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1142,6 +1168,11 @@
           <t>caster: Ball Lightning (sustained, mana-limited)</t>
         </is>
       </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1219,6 +1250,11 @@
           <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
         </is>
       </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1286,6 +1322,11 @@
           <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
         </is>
       </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1365,6 +1406,11 @@
           <t>caster: Chilly Bits Grade Peorth (sustained, mana-limited)</t>
         </is>
       </c>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1442,6 +1488,11 @@
           <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
         </is>
       </c>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1581,6 +1632,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV11" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1720,6 +1776,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1799,6 +1860,11 @@
           <t>caster: Super Shock (sustained, mana-limited)</t>
         </is>
       </c>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1878,6 +1944,11 @@
           <t>caster: Tsukikaze (sustained, mana-limited)</t>
         </is>
       </c>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1940,6 +2011,11 @@
           <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
         </is>
       </c>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2005,6 +2081,11 @@
           <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
         </is>
       </c>
+      <c r="AV16" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2070,6 +2151,11 @@
           <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
         </is>
       </c>
+      <c r="AV17" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2135,9 +2221,14 @@
           <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
         </is>
       </c>
+      <c r="AV18" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AU18"/>
+  <autoFilter ref="A1:AV18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5551,7 +5642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV15"/>
+  <dimension ref="A1:AW15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5602,6 +5693,7 @@
     <col width="17" customWidth="1" min="46" max="46"/>
     <col width="27" customWidth="1" min="47" max="47"/>
     <col width="14" customWidth="1" min="48" max="48"/>
+    <col width="13" customWidth="1" min="49" max="49"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5845,6 +5937,11 @@
           <t>dps_source</t>
         </is>
       </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>cost_source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5968,6 +6065,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6081,6 +6183,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AW3" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6194,6 +6301,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AW4" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6307,6 +6419,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AW5" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6420,6 +6537,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AW6" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6533,6 +6655,11 @@
       <c r="AV7" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="AW7" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -6658,6 +6785,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AW8" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -6798,6 +6930,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AW9" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6916,6 +7053,11 @@
       <c r="AV10" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="AW10" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -7041,6 +7183,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AW11" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7164,6 +7311,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7302,6 +7454,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AW13" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7440,6 +7597,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AW14" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7565,9 +7727,14 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AW15" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AV15"/>
+  <autoFilter ref="A1:AW15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7578,7 +7745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU20"/>
+  <dimension ref="A1:AV20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7628,6 +7795,7 @@
     <col width="15" customWidth="1" min="45" max="45"/>
     <col width="22" customWidth="1" min="46" max="46"/>
     <col width="14" customWidth="1" min="47" max="47"/>
+    <col width="13" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7866,6 +8034,11 @@
           <t>dps_source</t>
         </is>
       </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>cost_source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8005,6 +8178,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8144,6 +8322,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8288,6 +8471,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8429,6 +8617,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8570,6 +8763,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8709,6 +8907,11 @@
       <c r="AU7" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -8850,6 +9053,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -8984,6 +9192,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9128,6 +9341,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9272,6 +9490,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV11" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9411,6 +9634,11 @@
       <c r="AU12" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -9557,6 +9785,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9696,6 +9929,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -9835,6 +10073,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9976,6 +10219,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV16" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -10117,6 +10365,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV17" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -10258,6 +10511,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV18" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -10394,6 +10652,11 @@
       <c r="AU19" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="AV19" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -10540,9 +10803,14 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV20" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AU20"/>
+  <autoFilter ref="A1:AV20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10553,7 +10821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA28"/>
+  <dimension ref="A1:BB28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -10609,6 +10877,7 @@
     <col width="15" customWidth="1" min="51" max="51"/>
     <col width="22" customWidth="1" min="52" max="52"/>
     <col width="48" customWidth="1" min="53" max="53"/>
+    <col width="48" customWidth="1" min="54" max="54"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10877,6 +11146,11 @@
           <t>dps_source</t>
         </is>
       </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>cost_source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -11016,6 +11290,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -11165,6 +11444,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -11179,6 +11463,9 @@
       </c>
       <c r="C4" t="n">
         <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>80</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -11276,6 +11563,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB4" t="inlineStr">
+        <is>
+          <t>owner read in game 2026-09-12; the map sets no gold cost for this unit</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -11417,6 +11709,11 @@
       <c r="BA5" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="BB5" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -11573,6 +11870,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -11709,6 +12011,11 @@
       <c r="BA7" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -11892,6 +12199,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12041,6 +12353,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12195,6 +12512,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB10" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -12346,6 +12668,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB11" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -12495,6 +12822,11 @@
       <c r="BA12" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -12641,6 +12973,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB13" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -12790,6 +13127,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB14" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -12944,6 +13286,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB15" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -13098,6 +13445,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB16" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -13242,6 +13594,11 @@
       <c r="BA17" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="BB17" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -13388,6 +13745,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB18" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -13529,6 +13891,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB19" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -13673,6 +14040,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB20" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -13812,6 +14184,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB21" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -13988,6 +14365,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB22" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -14313,7 +14695,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BA28"/>
+  <autoFilter ref="A1:BB28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14324,7 +14706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU21"/>
+  <dimension ref="A1:AV21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -14374,6 +14756,7 @@
     <col width="15" customWidth="1" min="45" max="45"/>
     <col width="22" customWidth="1" min="46" max="46"/>
     <col width="48" customWidth="1" min="47" max="47"/>
+    <col width="13" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14612,6 +14995,11 @@
           <t>dps_source</t>
         </is>
       </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>cost_source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -14746,6 +15134,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -14880,6 +15273,11 @@
       <c r="AU3" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -15026,6 +15424,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -15110,6 +15513,11 @@
           <t>caster: Foxfire Laser (sustained, mana-limited)</t>
         </is>
       </c>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -15254,6 +15662,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -15398,6 +15811,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -15532,6 +15950,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -15671,6 +16094,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -15815,6 +16243,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -15959,6 +16392,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV11" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -16043,6 +16481,11 @@
           <t>caster: Fury of the Gods (sustained, mana-limited)</t>
         </is>
       </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -16182,6 +16625,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -16323,6 +16771,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -16464,6 +16917,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -16608,6 +17066,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV16" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -16752,6 +17215,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV17" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -16891,6 +17359,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV18" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -17027,6 +17500,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV19" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -17166,6 +17644,11 @@
       <c r="AU20" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="AV20" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -17307,9 +17790,14 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AV21" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AU21"/>
+  <autoFilter ref="A1:AV21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17320,7 +17808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY24"/>
+  <dimension ref="A1:AZ24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -17374,6 +17862,7 @@
     <col width="15" customWidth="1" min="49" max="49"/>
     <col width="22" customWidth="1" min="50" max="50"/>
     <col width="48" customWidth="1" min="51" max="51"/>
+    <col width="13" customWidth="1" min="52" max="52"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -17632,6 +18121,11 @@
           <t>dps_source</t>
         </is>
       </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>cost_source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -17786,6 +18280,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -17940,6 +18439,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -18091,6 +18595,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -18232,6 +18741,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -18380,6 +18894,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -18526,6 +19045,11 @@
       <c r="AY7" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -18669,6 +19193,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -18813,6 +19342,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -18967,6 +19501,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AZ10" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -19121,6 +19660,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AZ11" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -19270,6 +19814,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AZ12" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -19421,6 +19970,11 @@
       <c r="AY13" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="AZ13" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -19586,6 +20140,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AZ14" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -19740,6 +20299,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AZ15" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -19894,6 +20458,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AZ16" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -20048,6 +20617,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AZ17" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -20197,6 +20771,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AZ18" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -20351,6 +20930,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AZ19" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -20495,6 +21079,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AZ20" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -20724,7 +21313,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AY24"/>
+  <autoFilter ref="A1:AZ24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20735,7 +21324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA22"/>
+  <dimension ref="A1:BB22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -20791,6 +21380,7 @@
     <col width="15" customWidth="1" min="51" max="51"/>
     <col width="22" customWidth="1" min="52" max="52"/>
     <col width="48" customWidth="1" min="53" max="53"/>
+    <col width="13" customWidth="1" min="54" max="54"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -21059,6 +21649,11 @@
           <t>dps_source</t>
         </is>
       </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>cost_source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -21213,6 +21808,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -21362,6 +21962,11 @@
       <c r="BA3" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -21518,6 +22123,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB4" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -21672,6 +22282,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB5" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -21821,6 +22436,11 @@
       <c r="BA6" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -21972,6 +22592,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -22121,6 +22746,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -22270,6 +22900,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -22424,6 +23059,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB10" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -22604,6 +23244,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB11" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -22755,6 +23400,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -22904,6 +23554,11 @@
       <c r="BA13" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="BB13" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -23055,6 +23710,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB14" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -23206,6 +23866,11 @@
       <c r="BA15" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="BB15" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -23297,6 +23962,11 @@
           <t>caster: Thresh Arrow (sustained, mana-limited)</t>
         </is>
       </c>
+      <c r="BB16" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -23446,6 +24116,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB17" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -23627,6 +24302,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB18" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -23773,6 +24453,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="BB19" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -23938,6 +24623,11 @@
       <c r="BA20" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="BB20" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -24058,7 +24748,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BA22"/>
+  <autoFilter ref="A1:BB22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -40060,16 +40750,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C2" t="n">
-        <v>3.14</v>
+        <v>2.75</v>
       </c>
       <c r="D2" t="n">
         <v>1300</v>
       </c>
       <c r="E2" t="n">
-        <v>9.31</v>
+        <v>8.56</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -40096,16 +40786,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" t="n">
-        <v>5.87</v>
+        <v>5.78</v>
       </c>
       <c r="D3" t="n">
         <v>700</v>
       </c>
       <c r="E3" t="n">
-        <v>6.52</v>
+        <v>7.26</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -40128,34 +40818,34 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>tempest</t>
+          <t>ranger</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C4" t="n">
-        <v>4.12</v>
+        <v>5.11</v>
       </c>
       <c r="D4" t="n">
-        <v>850</v>
+        <v>800</v>
       </c>
       <c r="E4" t="n">
-        <v>5.84</v>
+        <v>5.82</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Jenovaroth</t>
+          <t>Noir Heart</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>800</v>
+        <v>415</v>
       </c>
       <c r="H4" t="n">
-        <v>101.08</v>
+        <v>68.42</v>
       </c>
       <c r="I4" t="n">
-        <v>21686</v>
+        <v>14924</v>
       </c>
       <c r="J4" t="n">
         <v>5</v>
@@ -40164,34 +40854,34 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ranger</t>
+          <t>tempest</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>19</v>
       </c>
       <c r="C5" t="n">
-        <v>5.11</v>
+        <v>4.08</v>
       </c>
       <c r="D5" t="n">
         <v>800</v>
       </c>
       <c r="E5" t="n">
-        <v>5.82</v>
+        <v>5.22</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Noir Heart</t>
+          <t>Jenovaroth</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>415</v>
+        <v>800</v>
       </c>
       <c r="H5" t="n">
-        <v>68.42</v>
+        <v>101.08</v>
       </c>
       <c r="I5" t="n">
-        <v>14924</v>
+        <v>21686</v>
       </c>
       <c r="J5" t="n">
         <v>5</v>
@@ -40240,16 +40930,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C7" t="n">
-        <v>2.47</v>
+        <v>2.05</v>
       </c>
       <c r="D7" t="n">
         <v>725</v>
       </c>
       <c r="E7" t="n">
-        <v>3.24</v>
+        <v>2.82</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -41714,7 +42404,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX20"/>
+  <dimension ref="A1:AY20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -41767,6 +42457,7 @@
     <col width="15" customWidth="1" min="48" max="48"/>
     <col width="22" customWidth="1" min="49" max="49"/>
     <col width="14" customWidth="1" min="50" max="50"/>
+    <col width="13" customWidth="1" min="51" max="51"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -42020,6 +42711,11 @@
           <t>dps_source</t>
         </is>
       </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>cost_source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -42154,6 +42850,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -42288,6 +42989,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -42424,6 +43130,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -42558,6 +43269,11 @@
       <c r="AX5" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -42699,6 +43415,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -42843,6 +43564,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -42972,6 +43698,11 @@
       <c r="AX8" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -43103,6 +43834,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -43242,6 +43978,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -43381,6 +44122,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -43515,6 +44261,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -43646,6 +44397,11 @@
       <c r="AX13" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="AY13" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -43777,6 +44533,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -43913,6 +44674,11 @@
       <c r="AX15" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="AY15" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -44061,6 +44827,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AY16" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -44197,6 +44968,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AY17" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -44363,6 +45139,11 @@
       <c r="AX18" t="inlineStr">
         <is>
           <t>basic attack</t>
+        </is>
+      </c>
+      <c r="AY18" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -44496,6 +45277,11 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AY19" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -44630,9 +45416,14 @@
           <t>basic attack</t>
         </is>
       </c>
+      <c r="AY20" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AX20"/>
+  <autoFilter ref="A1:AY20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
hero_ranking regenerated from the champion CSVs rather than recomputed
It had been produced by a separate script with its own copy of the formulas, so it
drifted from the files it summarises when the damage model gained poison and Bash.
Now a pure aggregate. The order of the seven champions is unchanged.
</commit_message>
<xml_diff>
--- a/skibi-data.xlsx
+++ b/skibi-data.xlsx
@@ -35,7 +35,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'bosses'!$A$1:$O$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'caster_dps'!$A$1:$L$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'game_modes'!$A$1:$I$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'hero_ranking'!$A$1:$J$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'hero_ranking'!$A$1:$K$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'heroes'!$A$1:$H$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'military'!$A$1:$AY$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'minigame_items'!$A$1:$D$22</definedName>
@@ -10877,7 +10877,7 @@
     <col width="15" customWidth="1" min="51" max="51"/>
     <col width="22" customWidth="1" min="52" max="52"/>
     <col width="48" customWidth="1" min="53" max="53"/>
-    <col width="48" customWidth="1" min="54" max="54"/>
+    <col width="13" customWidth="1" min="54" max="54"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11565,7 +11565,7 @@
       </c>
       <c r="BB4" t="inlineStr">
         <is>
-          <t>owner read in game 2026-09-12; the map sets no gold cost for this unit</t>
+          <t>map</t>
         </is>
       </c>
     </row>
@@ -40676,19 +40676,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="29" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="29" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -40699,45 +40700,50 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>towers</t>
+          <t>towers_scored</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>towers_total</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>median_dps_per_gold</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>median_range</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>median_coverage_adj_eff</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>best_tower</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>best_tower_cost</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>best_tower_coverage_adj_eff</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>peak_dps</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>hero_abilities</t>
         </is>
@@ -40753,29 +40759,32 @@
         <v>20</v>
       </c>
       <c r="C2" t="n">
-        <v>2.75</v>
+        <v>20</v>
       </c>
       <c r="D2" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E2" t="n">
         <v>1300</v>
       </c>
-      <c r="E2" t="n">
-        <v>8.56</v>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>Glacial Spike</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>935</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>45.85</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>13333</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -40789,29 +40798,32 @@
         <v>21</v>
       </c>
       <c r="C3" t="n">
-        <v>5.78</v>
+        <v>27</v>
       </c>
       <c r="D3" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="E3" t="n">
         <v>700</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>7.26</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Martyr</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>260</v>
       </c>
-      <c r="H3" t="n">
-        <v>41.27</v>
-      </c>
       <c r="I3" t="n">
-        <v>6963</v>
+        <v>41.86</v>
       </c>
       <c r="J3" t="n">
+        <v>7063</v>
+      </c>
+      <c r="K3" t="n">
         <v>5</v>
       </c>
     </row>
@@ -40825,29 +40837,32 @@
         <v>19</v>
       </c>
       <c r="C4" t="n">
-        <v>5.11</v>
+        <v>19</v>
       </c>
       <c r="D4" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="E4" t="n">
         <v>800</v>
       </c>
-      <c r="E4" t="n">
-        <v>5.82</v>
-      </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" t="n">
+        <v>5.84</v>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>Noir Heart</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>415</v>
       </c>
-      <c r="H4" t="n">
-        <v>68.42</v>
-      </c>
       <c r="I4" t="n">
-        <v>14924</v>
+        <v>68.58</v>
       </c>
       <c r="J4" t="n">
+        <v>14960</v>
+      </c>
+      <c r="K4" t="n">
         <v>5</v>
       </c>
     </row>
@@ -40861,101 +40876,110 @@
         <v>19</v>
       </c>
       <c r="C5" t="n">
-        <v>4.08</v>
+        <v>21</v>
       </c>
       <c r="D5" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>850</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5.84</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Jenovaroth</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
         <v>800</v>
       </c>
-      <c r="E5" t="n">
-        <v>5.22</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Jenovaroth</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>800</v>
-      </c>
-      <c r="H5" t="n">
-        <v>101.08</v>
-      </c>
       <c r="I5" t="n">
-        <v>21686</v>
+        <v>101.25</v>
       </c>
       <c r="J5" t="n">
+        <v>21722</v>
+      </c>
+      <c r="K5" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>specialist</t>
+          <t>arcane</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="C6" t="n">
-        <v>4.41</v>
+        <v>17</v>
       </c>
       <c r="D6" t="n">
-        <v>800</v>
+        <v>2.04</v>
       </c>
       <c r="E6" t="n">
-        <v>5.09</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Apocalypse</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>800</v>
+        <v>1150</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5.43</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Fire Hydra</t>
+        </is>
       </c>
       <c r="H6" t="n">
-        <v>28.28</v>
+        <v>255</v>
       </c>
       <c r="I6" t="n">
-        <v>7036</v>
+        <v>6.41</v>
       </c>
       <c r="J6" t="n">
+        <v>1357</v>
+      </c>
+      <c r="K6" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>arcane</t>
+          <t>specialist</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="C7" t="n">
-        <v>2.05</v>
+        <v>23</v>
       </c>
       <c r="D7" t="n">
-        <v>725</v>
+        <v>4.41</v>
       </c>
       <c r="E7" t="n">
-        <v>2.82</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Fire Hydra</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>255</v>
+        <v>800</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Apocalypse</t>
+        </is>
       </c>
       <c r="H7" t="n">
-        <v>6.41</v>
+        <v>800</v>
       </c>
       <c r="I7" t="n">
-        <v>1357</v>
+        <v>28.28</v>
       </c>
       <c r="J7" t="n">
+        <v>7036</v>
+      </c>
+      <c r="K7" t="n">
         <v>5</v>
       </c>
     </row>
@@ -40969,34 +40993,37 @@
         <v>19</v>
       </c>
       <c r="C8" t="n">
+        <v>19</v>
+      </c>
+      <c r="D8" t="n">
         <v>9.59</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>125</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>0.59</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Tamed Game</t>
         </is>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>205</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>20.54</v>
       </c>
-      <c r="I8" t="n">
-        <v>8932</v>
-      </c>
       <c r="J8" t="n">
+        <v>9026</v>
+      </c>
+      <c r="K8" t="n">
         <v>5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J8"/>
+  <autoFilter ref="A1:K8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Merge hand-captured rows onto the towers they describe
Six towers were spelled differently in the play capture and the map, so the join
failed and their notes sat as duplicate rows — Royal Family read as 27 towers
instead of 22. Merged by explicit pairing, not fuzzy matching (a fuzzy pass wrongly
proposed Father Dragon => Death Dragon; Father Dragon is its own unit).
</commit_message>
<xml_diff>
--- a/skibi-data.xlsx
+++ b/skibi-data.xlsx
@@ -43,9 +43,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'minigames'!$A$1:$I$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'other_towers'!$A$1:$AW$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'ranger'!$A$1:$AV$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'royal_family'!$A$1:$BB$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'royal_family'!$A$1:$BC$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'scarlet_knight'!$A$1:$AV$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'specialist'!$A$1:$AZ$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'specialist'!$A$1:$BA$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'tempest'!$A$1:$BB$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'tower_traits'!$A$1:$I$113</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'wave_modifiers'!$A$1:$D$46</definedName>
@@ -10821,7 +10821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB28"/>
+  <dimension ref="A1:BC23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -10878,6 +10878,7 @@
     <col width="22" customWidth="1" min="52" max="52"/>
     <col width="48" customWidth="1" min="53" max="53"/>
     <col width="13" customWidth="1" min="54" max="54"/>
+    <col width="21" customWidth="1" min="55" max="55"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11151,6 +11152,11 @@
           <t>cost_source</t>
         </is>
       </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>hand_capture_name</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -11251,6 +11257,16 @@
       <c r="AJ2" t="inlineStr">
         <is>
           <t>Build Grayson's Fort Buster ( R )</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>observed</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>COSTS 1 FOOD - a THIRD resource beyond gold and tiles, capped at 5 and unlocked partway through the run. So gold is not its real cost: at 175g it is the best gold-efficiency in the kit after Odin's Soul, but you can field at most FIVE food towers all run, and it competes against every other food tower rather than against 175g of anything else. SIEGE, so 13.82 becomes 22.11 on the Fortified waves (3, 8, 13, 18). Wave-20 gated.</t>
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
@@ -11295,6 +11311,11 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>Grayson Fort Buster</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -11670,6 +11691,21 @@
           <t>Build Tyr's Spirit ( W )</t>
         </is>
       </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>observed</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>Unlock confirmed by the owner 2026-09-05. BOUGHT FOR THE STUN, NOT THE DAMAGE. At very rapid fire a 20% proc lands every ~1.75s and the stun lasts 1.5s, so it holds ~86% STUN UPTIME on non-hero ground units - near-permanent lockdown. Damage is a modest 3.63 range-adjusted. BASH is a named tier trait: the treant Battleship Mackinaw carries a higher one (20%, +235, 2.0s, non-boss) - same 20% chance and same shape, and its "non-boss" is the same exclusion as this one's "non-hero".</t>
+        </is>
+      </c>
       <c r="AQ5" s="2" t="n">
         <v>388</v>
       </c>
@@ -11714,6 +11750,11 @@
       <c r="BB5" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="BC5" t="inlineStr">
+        <is>
+          <t>Tyr Spirit</t>
         </is>
       </c>
     </row>
@@ -11974,6 +12015,16 @@
           <t>Build Peppy Bronzebeard ( E )</t>
         </is>
       </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>observed</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>NO CRIT - untyped damage, so its 8.33 applies on EVERY wave rather than on a schedule, unlike most elite towers here. SLOW POISON III is the headline: 260 dps and 65% slow. The 260 dps alone out-damages several whole towers (treant Machination 54 dps, hawk Lasher 74 dps), so at tier III a debuff is worth more than a cheap tower. Completes the Slow Poison curve: 4 -&gt; 36 -&gt; 260 dps, 25% -&gt; 40% -&gt; 65% slow.</t>
+        </is>
+      </c>
       <c r="AQ7" s="2" t="n">
         <v>1485</v>
       </c>
@@ -12016,6 +12067,11 @@
       <c r="BB7" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="BC7" t="inlineStr">
+        <is>
+          <t>Peepy Bronzebeard</t>
         </is>
       </c>
     </row>
@@ -12936,6 +12992,16 @@
           <t>Build Petrified Cell ( C )</t>
         </is>
       </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>observed</t>
+        </is>
+      </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>THE K-DIG LINE ENDS IN A TANK. 3.22 range-adjusted is low, but FORTITUDE is durability + splash and eff/g cannot see survivability - the same caveat as the treant Ruby Scorpion, and a tower that dies is worth 0. Note the line's arc: K-Dig (siege utility/heal) -&gt; Xavier (siege damage) -&gt; Bartlebee (stun) -&gt; Delphinus (mana + spells) -&gt; this (tank). FIVE different jobs down one line. TWO NEW TRAITS: FROST I (the treant Sewage Surprise carries an unlabelled "frost", so that is probably the same family) and FORTITUDE. FAST = RAPID confirmed by the owner 2026-09-05, so the five bands stand.</t>
+        </is>
+      </c>
       <c r="AQ13" s="2" t="n">
         <v>600</v>
       </c>
@@ -12978,6 +13044,11 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC13" t="inlineStr">
+        <is>
+          <t>Petrified Shell</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -14147,6 +14218,16 @@
           <t>Build Lilianna Mai ( F )</t>
         </is>
       </c>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>observed</t>
+        </is>
+      </c>
+      <c r="AP21" t="inlineStr">
+        <is>
+          <t>CORRECTED 2026-09-05: damage is 1000-1455 (a normal 1.46x roll), not 100-1455. An earlier note here called it the widest spread recorded and read it as a deliberately unreliable autoattack - that was built on the typo and is WITHDRAWN. At 5.12 range-adjusted it is still modest for 850g plus a food slot, so it is still bought for its spells, but by the ordinary reading rather than a variance argument. GRAVITY WELL CORRECTED: 10% of LIFE as damage plus a 5% PERMANENT speed reduction - double the damage I first recorded, and a smaller but PERMANENT slow. "Permanent" implies it may STACK across casts, which would make it a different mechanic class from every other slow here. Worth confirming whether it stacks. DIVINE SHIELD makes the TOWER immune for 10s, the answer to the tower-destroying boss the owner flagged in their first message. Priciest Royal Family tower AND food-capped.</t>
+        </is>
+      </c>
       <c r="AQ21" s="2" t="n">
         <v>4910</v>
       </c>
@@ -14189,6 +14270,11 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC21" t="inlineStr">
+        <is>
+          <t>Lilliana May</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -14374,7 +14460,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Tyr Spirit</t>
+          <t>Royal Base II</t>
         </is>
       </c>
       <c r="AA23" s="2" t="n"/>
@@ -14383,14 +14469,9 @@
           <t>hand capture only — no extracted counterpart</t>
         </is>
       </c>
-      <c r="AO23" t="inlineStr">
-        <is>
-          <t>D3</t>
-        </is>
-      </c>
       <c r="AP23" t="inlineStr">
         <is>
-          <t>Unlock confirmed by the owner 2026-09-05. BOUGHT FOR THE STUN, NOT THE DAMAGE. At very rapid fire a 20% proc lands every ~1.75s and the stun lasts 1.5s, so it holds ~86% STUN UPTIME on non-hero ground units - near-permanent lockdown. Damage is a modest 3.63 range-adjusted. BASH is a named tier trait: the treant Battleship Mackinaw carries a higher one (20%, +235, 2.0s, non-boss) - same 20% chance and same shape, and its "non-boss" is the same exclusion as this one's "non-hero".</t>
+          <t>NOT A TOWER and not a "base tower" either - it is an upgrade purchased at the HERO SELECTION BUILDING (owner 2026-09-05). At 50g it is a pure tech gate for Peepy Bronzebeard, Cloud Buster, Lilliana May and Petrified Shell. It has no stat block to collect. The mechanism is per-hero: the Tempest Hawk has no equivalent.</t>
         </is>
       </c>
       <c r="AQ23" s="2" t="n"/>
@@ -14429,273 +14510,8 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Royal Base II</t>
-        </is>
-      </c>
-      <c r="AA24" s="2" t="n"/>
-      <c r="AN24" t="inlineStr">
-        <is>
-          <t>hand capture only — no extracted counterpart</t>
-        </is>
-      </c>
-      <c r="AP24" t="inlineStr">
-        <is>
-          <t>NOT A TOWER and not a "base tower" either - it is an upgrade purchased at the HERO SELECTION BUILDING (owner 2026-09-05). At 50g it is a pure tech gate for Peepy Bronzebeard, Cloud Buster, Lilliana May and Petrified Shell. It has no stat block to collect. The mechanism is per-hero: the Tempest Hawk has no equivalent.</t>
-        </is>
-      </c>
-      <c r="AQ24" s="2" t="n"/>
-      <c r="AR24" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS24" s="2">
-        <f>AQ24*AR24</f>
-        <v/>
-      </c>
-      <c r="AT24" s="3">
-        <f>IF(D24=0,"",AY24/D24)</f>
-        <v/>
-      </c>
-      <c r="AU24" s="3">
-        <f>(N24/725)^2</f>
-        <v/>
-      </c>
-      <c r="AV24" s="3">
-        <f>IF(D24=0,"",AT24*AU24)</f>
-        <v/>
-      </c>
-      <c r="AW24" s="2" t="n"/>
-      <c r="AX24" s="2" t="n"/>
-      <c r="AY24" s="2">
-        <f>AS24+N(AW24)+N(AX24)</f>
-        <v/>
-      </c>
-      <c r="AZ24" s="3">
-        <f>IF(D24=0,"",AT24*(N24/725))</f>
-        <v/>
-      </c>
-      <c r="BA24" t="inlineStr">
-        <is>
-          <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Peepy Bronzebeard</t>
-        </is>
-      </c>
-      <c r="AA25" s="2" t="n"/>
-      <c r="AN25" t="inlineStr">
-        <is>
-          <t>hand capture only — no extracted counterpart</t>
-        </is>
-      </c>
-      <c r="AP25" t="inlineStr">
-        <is>
-          <t>NO CRIT - untyped damage, so its 8.33 applies on EVERY wave rather than on a schedule, unlike most elite towers here. SLOW POISON III is the headline: 260 dps and 65% slow. The 260 dps alone out-damages several whole towers (treant Machination 54 dps, hawk Lasher 74 dps), so at tier III a debuff is worth more than a cheap tower. Completes the Slow Poison curve: 4 -&gt; 36 -&gt; 260 dps, 25% -&gt; 40% -&gt; 65% slow.</t>
-        </is>
-      </c>
-      <c r="AQ25" s="2" t="n"/>
-      <c r="AR25" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS25" s="2">
-        <f>AQ25*AR25</f>
-        <v/>
-      </c>
-      <c r="AT25" s="3">
-        <f>IF(D25=0,"",AY25/D25)</f>
-        <v/>
-      </c>
-      <c r="AU25" s="3">
-        <f>(N25/725)^2</f>
-        <v/>
-      </c>
-      <c r="AV25" s="3">
-        <f>IF(D25=0,"",AT25*AU25)</f>
-        <v/>
-      </c>
-      <c r="AW25" s="2" t="n"/>
-      <c r="AX25" s="2" t="n"/>
-      <c r="AY25" s="2">
-        <f>AS25+N(AW25)+N(AX25)</f>
-        <v/>
-      </c>
-      <c r="AZ25" s="3">
-        <f>IF(D25=0,"",AT25*(N25/725))</f>
-        <v/>
-      </c>
-      <c r="BA25" t="inlineStr">
-        <is>
-          <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Grayson Fort Buster</t>
-        </is>
-      </c>
-      <c r="AA26" s="2" t="n"/>
-      <c r="AN26" t="inlineStr">
-        <is>
-          <t>hand capture only — no extracted counterpart</t>
-        </is>
-      </c>
-      <c r="AP26" t="inlineStr">
-        <is>
-          <t>COSTS 1 FOOD - a THIRD resource beyond gold and tiles, capped at 5 and unlocked partway through the run. So gold is not its real cost: at 175g it is the best gold-efficiency in the kit after Odin's Soul, but you can field at most FIVE food towers all run, and it competes against every other food tower rather than against 175g of anything else. SIEGE, so 13.82 becomes 22.11 on the Fortified waves (3, 8, 13, 18). Wave-20 gated.</t>
-        </is>
-      </c>
-      <c r="AQ26" s="2" t="n"/>
-      <c r="AR26" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS26" s="2">
-        <f>AQ26*AR26</f>
-        <v/>
-      </c>
-      <c r="AT26" s="3">
-        <f>IF(D26=0,"",AY26/D26)</f>
-        <v/>
-      </c>
-      <c r="AU26" s="3">
-        <f>(N26/725)^2</f>
-        <v/>
-      </c>
-      <c r="AV26" s="3">
-        <f>IF(D26=0,"",AT26*AU26)</f>
-        <v/>
-      </c>
-      <c r="AW26" s="2" t="n"/>
-      <c r="AX26" s="2" t="n"/>
-      <c r="AY26" s="2">
-        <f>AS26+N(AW26)+N(AX26)</f>
-        <v/>
-      </c>
-      <c r="AZ26" s="3">
-        <f>IF(D26=0,"",AT26*(N26/725))</f>
-        <v/>
-      </c>
-      <c r="BA26" t="inlineStr">
-        <is>
-          <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Lilliana May</t>
-        </is>
-      </c>
-      <c r="AA27" s="2" t="n"/>
-      <c r="AN27" t="inlineStr">
-        <is>
-          <t>hand capture only — no extracted counterpart</t>
-        </is>
-      </c>
-      <c r="AP27" t="inlineStr">
-        <is>
-          <t>CORRECTED 2026-09-05: damage is 1000-1455 (a normal 1.46x roll), not 100-1455. An earlier note here called it the widest spread recorded and read it as a deliberately unreliable autoattack - that was built on the typo and is WITHDRAWN. At 5.12 range-adjusted it is still modest for 850g plus a food slot, so it is still bought for its spells, but by the ordinary reading rather than a variance argument. GRAVITY WELL CORRECTED: 10% of LIFE as damage plus a 5% PERMANENT speed reduction - double the damage I first recorded, and a smaller but PERMANENT slow. "Permanent" implies it may STACK across casts, which would make it a different mechanic class from every other slow here. Worth confirming whether it stacks. DIVINE SHIELD makes the TOWER immune for 10s, the answer to the tower-destroying boss the owner flagged in their first message. Priciest Royal Family tower AND food-capped.</t>
-        </is>
-      </c>
-      <c r="AQ27" s="2" t="n"/>
-      <c r="AR27" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS27" s="2">
-        <f>AQ27*AR27</f>
-        <v/>
-      </c>
-      <c r="AT27" s="3">
-        <f>IF(D27=0,"",AY27/D27)</f>
-        <v/>
-      </c>
-      <c r="AU27" s="3">
-        <f>(N27/725)^2</f>
-        <v/>
-      </c>
-      <c r="AV27" s="3">
-        <f>IF(D27=0,"",AT27*AU27)</f>
-        <v/>
-      </c>
-      <c r="AW27" s="2" t="n"/>
-      <c r="AX27" s="2" t="n"/>
-      <c r="AY27" s="2">
-        <f>AS27+N(AW27)+N(AX27)</f>
-        <v/>
-      </c>
-      <c r="AZ27" s="3">
-        <f>IF(D27=0,"",AT27*(N27/725))</f>
-        <v/>
-      </c>
-      <c r="BA27" t="inlineStr">
-        <is>
-          <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Petrified Shell</t>
-        </is>
-      </c>
-      <c r="AA28" s="2" t="n"/>
-      <c r="AN28" t="inlineStr">
-        <is>
-          <t>hand capture only — no extracted counterpart</t>
-        </is>
-      </c>
-      <c r="AP28" t="inlineStr">
-        <is>
-          <t>THE K-DIG LINE ENDS IN A TANK. 3.22 range-adjusted is low, but FORTITUDE is durability + splash and eff/g cannot see survivability - the same caveat as the treant Ruby Scorpion, and a tower that dies is worth 0. Note the line's arc: K-Dig (siege utility/heal) -&gt; Xavier (siege damage) -&gt; Bartlebee (stun) -&gt; Delphinus (mana + spells) -&gt; this (tank). FIVE different jobs down one line. TWO NEW TRAITS: FROST I (the treant Sewage Surprise carries an unlabelled "frost", so that is probably the same family) and FORTITUDE. FAST = RAPID confirmed by the owner 2026-09-05, so the five bands stand.</t>
-        </is>
-      </c>
-      <c r="AQ28" s="2" t="n"/>
-      <c r="AR28" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS28" s="2">
-        <f>AQ28*AR28</f>
-        <v/>
-      </c>
-      <c r="AT28" s="3">
-        <f>IF(D28=0,"",AY28/D28)</f>
-        <v/>
-      </c>
-      <c r="AU28" s="3">
-        <f>(N28/725)^2</f>
-        <v/>
-      </c>
-      <c r="AV28" s="3">
-        <f>IF(D28=0,"",AT28*AU28)</f>
-        <v/>
-      </c>
-      <c r="AW28" s="2" t="n"/>
-      <c r="AX28" s="2" t="n"/>
-      <c r="AY28" s="2">
-        <f>AS28+N(AW28)+N(AX28)</f>
-        <v/>
-      </c>
-      <c r="AZ28" s="3">
-        <f>IF(D28=0,"",AT28*(N28/725))</f>
-        <v/>
-      </c>
-      <c r="BA28" t="inlineStr">
-        <is>
-          <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:BB28"/>
+  <autoFilter ref="A1:BC23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17808,7 +17624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ24"/>
+  <dimension ref="A1:BA23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -17863,6 +17679,7 @@
     <col width="22" customWidth="1" min="50" max="50"/>
     <col width="48" customWidth="1" min="51" max="51"/>
     <col width="13" customWidth="1" min="52" max="52"/>
+    <col width="19" customWidth="1" min="53" max="53"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -18126,6 +17943,11 @@
           <t>cost_source</t>
         </is>
       </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>hand_capture_name</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -18704,6 +18526,21 @@
           <t>U pgrade to Gigas Spike</t>
         </is>
       </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>observed</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SIEGE (owner 2026-09-06) - note its BASE Spike Shooter is CHAOS, so this upgrade CHANGES type, the second confirmed case after Sewer Barge -&gt; Sewage Surprise. 4.95 becomes 7.92 on Fortified. RESOLVED 2026-09-05: the trait is named "Boss Assassin" but TARGETS HEROES - the owner read "boss assassin II (50% x8 against heroes)" on a Royal Family tower. So the earlier boss-vs-hero ambiguity was the GAME conflating them, not a transcription slip. Both readings were right. Upgrade of Spike Shooter. Keeps the anti-boss crit - 'same passive against boss', confirmed by the owner checking Giga Spikes directly (2026-09-03). Range jumps 600-&gt;900. </t>
+        </is>
+      </c>
       <c r="AO5" s="2" t="n">
         <v>477.8</v>
       </c>
@@ -18746,6 +18583,11 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BA5" t="inlineStr">
+        <is>
+          <t>Giga Spikes</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -21204,7 +21046,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Giga Spikes</t>
+          <t>Specialist Base</t>
         </is>
       </c>
       <c r="AA23" s="2" t="n"/>
@@ -21213,14 +21055,9 @@
           <t>hand capture only — no extracted counterpart</t>
         </is>
       </c>
-      <c r="AM23" t="inlineStr">
-        <is>
-          <t>D4</t>
-        </is>
-      </c>
       <c r="AN23" t="inlineStr">
         <is>
-          <t xml:space="preserve">SIEGE (owner 2026-09-06) - note its BASE Spike Shooter is CHAOS, so this upgrade CHANGES type, the second confirmed case after Sewer Barge -&gt; Sewage Surprise. 4.95 becomes 7.92 on Fortified. RESOLVED 2026-09-05: the trait is named "Boss Assassin" but TARGETS HEROES - the owner read "boss assassin II (50% x8 against heroes)" on a Royal Family tower. So the earlier boss-vs-hero ambiguity was the GAME conflating them, not a transcription slip. Both readings were right. Upgrade of Spike Shooter. Keeps the anti-boss crit - 'same passive against boss', confirmed by the owner checking Giga Spikes directly (2026-09-03). Range jumps 600-&gt;900. </t>
+          <t>THE TREANT HAS A BASE UPGRADE TOO. Analogous to the Royal Family's Royal Base II, which is bought at the hero-selection building. So base upgrades are present in 2 of 3 captured kits - the Tempest Hawk, which has none, is the exception. Cost and purchase location unread.</t>
         </is>
       </c>
       <c r="AO23" s="2" t="n"/>
@@ -21259,61 +21096,8 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Specialist Base</t>
-        </is>
-      </c>
-      <c r="AA24" s="2" t="n"/>
-      <c r="AL24" t="inlineStr">
-        <is>
-          <t>hand capture only — no extracted counterpart</t>
-        </is>
-      </c>
-      <c r="AN24" t="inlineStr">
-        <is>
-          <t>THE TREANT HAS A BASE UPGRADE TOO. Analogous to the Royal Family's Royal Base II, which is bought at the hero-selection building. So base upgrades are present in 2 of 3 captured kits - the Tempest Hawk, which has none, is the exception. Cost and purchase location unread.</t>
-        </is>
-      </c>
-      <c r="AO24" s="2" t="n"/>
-      <c r="AP24" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ24" s="2">
-        <f>AO24*AP24</f>
-        <v/>
-      </c>
-      <c r="AR24" s="3">
-        <f>IF(D24=0,"",AW24/D24)</f>
-        <v/>
-      </c>
-      <c r="AS24" s="3">
-        <f>(N24/725)^2</f>
-        <v/>
-      </c>
-      <c r="AT24" s="3">
-        <f>IF(D24=0,"",AR24*AS24)</f>
-        <v/>
-      </c>
-      <c r="AU24" s="2" t="n"/>
-      <c r="AV24" s="2" t="n"/>
-      <c r="AW24" s="2">
-        <f>AQ24+N(AU24)+N(AV24)</f>
-        <v/>
-      </c>
-      <c r="AX24" s="3">
-        <f>IF(D24=0,"",AR24*(N24/725))</f>
-        <v/>
-      </c>
-      <c r="AY24" t="inlineStr">
-        <is>
-          <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:AZ24"/>
+  <autoFilter ref="A1:BA23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -40798,7 +40582,7 @@
         <v>21</v>
       </c>
       <c r="C3" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D3" t="n">
         <v>5.88</v>
@@ -40954,7 +40738,7 @@
         <v>19</v>
       </c>
       <c r="C7" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D7" t="n">
         <v>4.41</v>

</xml_diff>

<commit_message>
Four units moved from other_towers into their champion kits
Sewage Surprise and Brahma's Fix-it Shop to specialist; Father Dragon and
Reaperspawn to tempest. They were in other_towers only because the older combined
extraction had no hero column; the hand capture names the kit for each, and moving
them also attaches the note that had been stranded. Play-note coverage for the
three hand-captured heroes is now 21/21, 19/20 and 19/20.
</commit_message>
<xml_diff>
--- a/skibi-data.xlsx
+++ b/skibi-data.xlsx
@@ -41,12 +41,12 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'minigame_items'!$A$1:$D$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'minigame_readings'!$A$1:$G$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'minigames'!$A$1:$I$80</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'other_towers'!$A$1:$AW$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'other_towers'!$A$1:$AW$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'ranger'!$A$1:$AV$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'royal_family'!$A$1:$BC$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'scarlet_knight'!$A$1:$AV$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'specialist'!$A$1:$BA$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'tempest'!$A$1:$BB$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'specialist'!$A$1:$BA$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'tempest'!$A$1:$BB$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'tower_traits'!$A$1:$I$113</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'wave_modifiers'!$A$1:$D$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'wave_traits'!$A$1:$K$51</definedName>
@@ -5642,11 +5642,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW15"/>
+  <dimension ref="A1:AW11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
@@ -5678,9 +5678,9 @@
     <col width="9" customWidth="1" min="31" max="31"/>
     <col width="26" customWidth="1" min="32" max="32"/>
     <col width="35" customWidth="1" min="33" max="33"/>
-    <col width="12" customWidth="1" min="34" max="34"/>
+    <col width="9" customWidth="1" min="34" max="34"/>
     <col width="17" customWidth="1" min="35" max="35"/>
-    <col width="48" customWidth="1" min="36" max="36"/>
+    <col width="11" customWidth="1" min="36" max="36"/>
     <col width="48" customWidth="1" min="37" max="37"/>
     <col width="9" customWidth="1" min="38" max="38"/>
     <col width="17" customWidth="1" min="39" max="39"/>
@@ -5946,60 +5946,55 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>h04H</t>
+          <t>h04I</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Brahma's Fix-it Shop</t>
+          <t>Equipped Peasant 1</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>95</v>
+        <v>10</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>175</v>
+        <v>19</v>
       </c>
       <c r="G2" t="n">
-        <v>175</v>
+        <v>21</v>
       </c>
       <c r="H2" t="n">
-        <v>175</v>
+        <v>20</v>
       </c>
       <c r="I2" t="n">
-        <v>1.5</v>
+        <v>0.6</v>
       </c>
       <c r="J2" t="n">
-        <v>116.7</v>
+        <v>33.3</v>
       </c>
       <c r="K2" t="n">
-        <v>1100</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>siege</t>
-        </is>
+        <v>125</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>missile</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>174</v>
+        <v>18</v>
       </c>
       <c r="O2" t="n">
         <v>1</v>
       </c>
       <c r="P2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>siege</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -6008,31 +6003,26 @@
         </is>
       </c>
       <c r="AD2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AE2" s="2" t="n">
-        <v>1500</v>
+        <v>1250</v>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>A03Y,A070,AChv,A028</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>Up g rade to Brahma's Fix-it Shop</t>
+          <t>A03C,A028</t>
         </is>
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>Machine Critical Strike (A03Y); Super Regeneration (A070); Empathic Fix (AChv); Sell Tower (A028)</t>
+          <t>Vindicator II (A03C); Sell Tower (A028)</t>
         </is>
       </c>
       <c r="AL2" s="2" t="n">
-        <v>116.7</v>
+        <v>33.3</v>
       </c>
       <c r="AM2" s="3" t="n">
-        <v>1.8</v>
+        <v>3.5</v>
       </c>
       <c r="AN2" s="2">
         <f>AL2*AM2</f>
@@ -6074,12 +6064,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>h04I</t>
+          <t>h03P</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Equipped Peasant 1</t>
+          <t>Equipped Peasant 2</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -6089,19 +6079,19 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" t="n">
+        <v>22</v>
+      </c>
+      <c r="H3" t="n">
         <v>21</v>
-      </c>
-      <c r="H3" t="n">
-        <v>20</v>
       </c>
       <c r="I3" t="n">
         <v>0.6</v>
       </c>
       <c r="J3" t="n">
-        <v>33.3</v>
+        <v>35</v>
       </c>
       <c r="K3" t="n">
         <v>125</v>
@@ -6112,7 +6102,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O3" t="n">
         <v>1</v>
@@ -6134,20 +6124,20 @@
         <v>0</v>
       </c>
       <c r="AE3" s="2" t="n">
-        <v>1250</v>
+        <v>1500</v>
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>A03C,A028</t>
+          <t>A03C,A004,A028</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>Vindicator II (A03C); Sell Tower (A028)</t>
+          <t>Vindicator II (A03C); Versatile Critical Strike I (A004); Sell Tower (A028)</t>
         </is>
       </c>
       <c r="AL3" s="2" t="n">
-        <v>33.3</v>
+        <v>35</v>
       </c>
       <c r="AM3" s="3" t="n">
         <v>3.5</v>
@@ -6192,12 +6182,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>h03P</t>
+          <t>h04O</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Equipped Peasant 2</t>
+          <t>Equipped Peasant 3</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -6207,19 +6197,19 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G4" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="H4" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I4" t="n">
         <v>0.6</v>
       </c>
       <c r="J4" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="K4" t="n">
         <v>125</v>
@@ -6230,13 +6220,13 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="O4" t="n">
         <v>1</v>
       </c>
       <c r="P4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -6249,23 +6239,23 @@
         </is>
       </c>
       <c r="AD4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE4" s="2" t="n">
-        <v>1500</v>
+        <v>1750</v>
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>A03C,A004,A028</t>
+          <t>A03C,A01E,A028</t>
         </is>
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>Vindicator II (A03C); Versatile Critical Strike I (A004); Sell Tower (A028)</t>
+          <t>Vindicator II (A03C); Versatile Critical Strike II (A01E); Sell Tower (A028)</t>
         </is>
       </c>
       <c r="AL4" s="2" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="AM4" s="3" t="n">
         <v>3.5</v>
@@ -6310,12 +6300,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>h04O</t>
+          <t>h04P</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Equipped Peasant 3</t>
+          <t>Equipped Peasant 4</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -6325,19 +6315,19 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G5" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="H5" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="I5" t="n">
         <v>0.6</v>
       </c>
       <c r="J5" t="n">
-        <v>40</v>
+        <v>46.7</v>
       </c>
       <c r="K5" t="n">
         <v>125</v>
@@ -6348,13 +6338,13 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="O5" t="n">
         <v>1</v>
       </c>
       <c r="P5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -6367,26 +6357,26 @@
         </is>
       </c>
       <c r="AD5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE5" s="2" t="n">
-        <v>1750</v>
+        <v>2000</v>
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>A03C,A01E,A028</t>
+          <t>A02Z,A01E,A028</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>Vindicator II (A03C); Versatile Critical Strike II (A01E); Sell Tower (A028)</t>
+          <t>Vindicator III (A02Z); Versatile Critical Strike II (A01E); Sell Tower (A028)</t>
         </is>
       </c>
       <c r="AL5" s="2" t="n">
-        <v>40</v>
+        <v>46.7</v>
       </c>
       <c r="AM5" s="3" t="n">
-        <v>3.5</v>
+        <v>5.5</v>
       </c>
       <c r="AN5" s="2">
         <f>AL5*AM5</f>
@@ -6428,12 +6418,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>h04P</t>
+          <t>h04Q</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Equipped Peasant 4</t>
+          <t>Equipped Peasant 5</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -6443,19 +6433,19 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="G6" t="n">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="H6" t="n">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="I6" t="n">
         <v>0.6</v>
       </c>
       <c r="J6" t="n">
-        <v>46.7</v>
+        <v>71.7</v>
       </c>
       <c r="K6" t="n">
         <v>125</v>
@@ -6466,13 +6456,13 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="O6" t="n">
         <v>1</v>
       </c>
       <c r="P6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -6485,23 +6475,23 @@
         </is>
       </c>
       <c r="AD6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AE6" s="2" t="n">
-        <v>2000</v>
+        <v>2250</v>
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>A02Z,A01E,A028</t>
+          <t>ANbh,A02Z,A01E,A028</t>
         </is>
       </c>
       <c r="AK6" t="inlineStr">
         <is>
-          <t>Vindicator III (A02Z); Versatile Critical Strike II (A01E); Sell Tower (A028)</t>
+          <t>Bash I (ANbh); Vindicator III (A02Z); Versatile Critical Strike II (A01E); Sell Tower (A028)</t>
         </is>
       </c>
       <c r="AL6" s="2" t="n">
-        <v>46.7</v>
+        <v>71.7</v>
       </c>
       <c r="AM6" s="3" t="n">
         <v>5.5</v>
@@ -6510,7 +6500,9 @@
         <f>AL6*AM6</f>
         <v/>
       </c>
-      <c r="AO6" s="2" t="n"/>
+      <c r="AO6" s="2" t="n">
+        <v>16.7</v>
+      </c>
       <c r="AP6" s="2" t="n"/>
       <c r="AQ6" s="2">
         <f>AN6+N(AO6)+N(AP6)</f>
@@ -6546,55 +6538,60 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>h04Q</t>
+          <t>h00R</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Equipped Peasant 5</t>
+          <t>Exiled Soul</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="G7" t="n">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="H7" t="n">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="I7" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="J7" t="n">
-        <v>71.7</v>
+        <v>280</v>
       </c>
       <c r="K7" t="n">
-        <v>125</v>
+        <v>600</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>chaos</t>
+        </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>missile</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="O7" t="n">
         <v>1</v>
       </c>
       <c r="P7" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>chaos</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -6603,34 +6600,37 @@
         </is>
       </c>
       <c r="AD7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AE7" s="2" t="n">
-        <v>2250</v>
+        <v>1500</v>
       </c>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>ANbh,A02Z,A01E,A028</t>
+          <t>A03W,A028,Afra</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>Up g rade to Exiled Soul</t>
         </is>
       </c>
       <c r="AK7" t="inlineStr">
         <is>
-          <t>Bash I (ANbh); Vindicator III (A02Z); Versatile Critical Strike II (A01E); Sell Tower (A028)</t>
+          <t>Regeneration (A03W); Sell Tower (A028); Frost I (Afra)</t>
         </is>
       </c>
       <c r="AL7" s="2" t="n">
-        <v>71.7</v>
+        <v>280</v>
       </c>
       <c r="AM7" s="3" t="n">
-        <v>5.5</v>
+        <v>1</v>
       </c>
       <c r="AN7" s="2">
         <f>AL7*AM7</f>
         <v/>
       </c>
-      <c r="AO7" s="2" t="n">
-        <v>16.7</v>
-      </c>
+      <c r="AO7" s="2" t="n"/>
       <c r="AP7" s="2" t="n"/>
       <c r="AQ7" s="2">
         <f>AN7+N(AO7)+N(AP7)</f>
@@ -6666,60 +6666,55 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>h00R</t>
+          <t>h00H</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Exiled Soul</t>
+          <t>Footman</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="G8" t="n">
-        <v>57</v>
+        <v>89</v>
       </c>
       <c r="H8" t="n">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="I8" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="J8" t="n">
-        <v>280</v>
+        <v>290</v>
       </c>
       <c r="K8" t="n">
-        <v>600</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>chaos</t>
-        </is>
+        <v>125</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>missile</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>54</v>
+        <v>84</v>
       </c>
       <c r="O8" t="n">
         <v>1</v>
       </c>
       <c r="P8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>chaos</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -6728,28 +6723,28 @@
         </is>
       </c>
       <c r="AD8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AE8" s="2" t="n">
-        <v>1500</v>
+        <v>1250</v>
       </c>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>A03W,A028,Afra</t>
+          <t>ANbh,A028</t>
         </is>
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>Up g rade to Exiled Soul</t>
+          <t>U pgrade to Footman</t>
         </is>
       </c>
       <c r="AK8" t="inlineStr">
         <is>
-          <t>Regeneration (A03W); Sell Tower (A028); Frost I (Afra)</t>
+          <t>Bash I (ANbh); Sell Tower (A028)</t>
         </is>
       </c>
       <c r="AL8" s="2" t="n">
-        <v>280</v>
+        <v>290</v>
       </c>
       <c r="AM8" s="3" t="n">
         <v>1</v>
@@ -6758,7 +6753,9 @@
         <f>AL8*AM8</f>
         <v/>
       </c>
-      <c r="AO8" s="2" t="n"/>
+      <c r="AO8" s="2" t="n">
+        <v>33.3</v>
+      </c>
       <c r="AP8" s="2" t="n"/>
       <c r="AQ8" s="2">
         <f>AN8+N(AO8)+N(AP8)</f>
@@ -6794,60 +6791,60 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>h01J</t>
+          <t>h03O</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Father Dragon</t>
+          <t>Heartseeker</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>298</v>
+        <v>23</v>
       </c>
       <c r="G9" t="n">
-        <v>298</v>
+        <v>28</v>
       </c>
       <c r="H9" t="n">
-        <v>298</v>
+        <v>25.5</v>
       </c>
       <c r="I9" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="J9" t="n">
-        <v>425.7</v>
+        <v>51</v>
       </c>
       <c r="K9" t="n">
-        <v>600</v>
+        <v>1150</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>magic</t>
+          <t>chaos</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>missile</t>
+          <t>instant</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>297</v>
+        <v>22</v>
       </c>
       <c r="O9" t="n">
         <v>1</v>
       </c>
       <c r="P9" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>magic</t>
+          <t>chaos</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -6863,48 +6860,31 @@
       </c>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>A03D,A028,A006,A008</t>
+          <t>Afbb,Aabr,AIva,A01E,A028</t>
         </is>
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>U pgrade to Father Dragon</t>
-        </is>
-      </c>
-      <c r="AH9" t="inlineStr">
-        <is>
-          <t>tempest</t>
-        </is>
-      </c>
-      <c r="AI9" t="inlineStr">
-        <is>
-          <t>D2</t>
-        </is>
-      </c>
-      <c r="AJ9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AIR CRITICAL STRIKE II identified 2026-09-05 (the Royal Family named the tier: 50% x4). RESOLVED 2026-09-05: the trait is named "Boss Assassin" but TARGETS HEROES - the owner read "boss assassin II (50% x8 against heroes)" on a Royal Family tower. So the earlier boss-vs-hero ambiguity was the GAME conflating them, not a transcription slip. Both readings were right. DUAL crit (air AND boss) at 50% x4 each. 16.78 range-adjusted against either. Its 600 range is short for the kit. </t>
+          <t>U pgrade to Heartseeker</t>
         </is>
       </c>
       <c r="AK9" t="inlineStr">
         <is>
-          <t>Boss Assassin I (A03D); Sell Tower (A028); Air Critical Strike II (A006); Slow Poison II (A008)</t>
+          <t>Sunder Armor (Afbb); (Dummy Ability - Life Steal) (Aabr); AIva (AIva); Versatile Critical Strike II (A01E); Sell Tower (A028)</t>
         </is>
       </c>
       <c r="AL9" s="2" t="n">
-        <v>425.7</v>
+        <v>51</v>
       </c>
       <c r="AM9" s="3" t="n">
-        <v>2.5</v>
+        <v>2.05</v>
       </c>
       <c r="AN9" s="2">
         <f>AL9*AM9</f>
         <v/>
       </c>
       <c r="AO9" s="2" t="n"/>
-      <c r="AP9" s="2" t="n">
-        <v>36</v>
-      </c>
+      <c r="AP9" s="2" t="n"/>
       <c r="AQ9" s="2">
         <f>AN9+N(AO9)+N(AP9)</f>
         <v/>
@@ -6939,55 +6919,63 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>h00H</t>
+          <t>h048</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Footman</t>
+          <t>Krotas</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>45</v>
+        <v>1325</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
       <c r="F10" t="n">
-        <v>85</v>
+        <v>851</v>
       </c>
       <c r="G10" t="n">
-        <v>89</v>
+        <v>858</v>
       </c>
       <c r="H10" t="n">
-        <v>87</v>
+        <v>854.5</v>
       </c>
       <c r="I10" t="n">
-        <v>0.3</v>
+        <v>0.33</v>
       </c>
       <c r="J10" t="n">
-        <v>290</v>
+        <v>2589.4</v>
       </c>
       <c r="K10" t="n">
-        <v>125</v>
+        <v>1500</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>chaos</t>
+        </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>missile</t>
         </is>
       </c>
       <c r="N10" t="n">
-        <v>84</v>
+        <v>850</v>
       </c>
       <c r="O10" t="n">
         <v>1</v>
       </c>
       <c r="P10" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>chaos</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -6995,40 +6983,35 @@
           <t>hhou</t>
         </is>
       </c>
-      <c r="AD10" t="n">
-        <v>1</v>
-      </c>
       <c r="AE10" s="2" t="n">
-        <v>1250</v>
+        <v>2500</v>
       </c>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>ANbh,A028</t>
+          <t>ANcl,A004,A02X,A014,A028</t>
         </is>
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>U pgrade to Footman</t>
+          <t>Up g rade to Krotas - 1325</t>
         </is>
       </c>
       <c r="AK10" t="inlineStr">
         <is>
-          <t>Bash I (ANbh); Sell Tower (A028)</t>
+          <t>Activate / Deactivate Mana Detection (ANcl); Versatile Critical Strike I (A004); Gooify (A02X); Combustion (A014); Sell Tower (A028)</t>
         </is>
       </c>
       <c r="AL10" s="2" t="n">
-        <v>290</v>
+        <v>2589.4</v>
       </c>
       <c r="AM10" s="3" t="n">
-        <v>1</v>
+        <v>1.52</v>
       </c>
       <c r="AN10" s="2">
         <f>AL10*AM10</f>
         <v/>
       </c>
-      <c r="AO10" s="2" t="n">
-        <v>33.3</v>
-      </c>
+      <c r="AO10" s="2" t="n"/>
       <c r="AP10" s="2" t="n"/>
       <c r="AQ10" s="2">
         <f>AN10+N(AO10)+N(AP10)</f>
@@ -7064,34 +7047,37 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>h03O</t>
+          <t>h047</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Heartseeker</t>
+          <t>Von Chillspeak</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>45</v>
+        <v>1225</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
       <c r="F11" t="n">
-        <v>23</v>
+        <v>12000</v>
       </c>
       <c r="G11" t="n">
-        <v>28</v>
+        <v>12000</v>
       </c>
       <c r="H11" t="n">
-        <v>25.5</v>
+        <v>12000</v>
       </c>
       <c r="I11" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="J11" t="n">
-        <v>51</v>
+        <v>6000</v>
       </c>
       <c r="K11" t="n">
         <v>1150</v>
@@ -7103,17 +7089,17 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>instant</t>
+          <t>missile</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>22</v>
+        <v>11999</v>
       </c>
       <c r="O11" t="n">
         <v>1</v>
       </c>
       <c r="P11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -7125,39 +7111,38 @@
           <t>hhou</t>
         </is>
       </c>
-      <c r="AD11" t="n">
-        <v>2</v>
-      </c>
       <c r="AE11" s="2" t="n">
-        <v>1500</v>
+        <v>2500</v>
       </c>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>Afbb,Aabr,AIva,A01E,A028</t>
+          <t>ANcl,Afrz,Aap1,AIm2,A028</t>
         </is>
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>U pgrade to Heartseeker</t>
+          <t>U pgrade to Von Chillspeak - 1225</t>
         </is>
       </c>
       <c r="AK11" t="inlineStr">
         <is>
-          <t>Sunder Armor (Afbb); (Dummy Ability - Life Steal) (Aabr); AIva (AIva); Versatile Critical Strike II (A01E); Sell Tower (A028)</t>
+          <t>Activate / Deactivate Mana Detection (ANcl); Stone Cold (Afrz); Grounding Curse (Aap1); Cold Snap (AIm2); Sell Tower (A028)</t>
         </is>
       </c>
       <c r="AL11" s="2" t="n">
-        <v>51</v>
+        <v>6000</v>
       </c>
       <c r="AM11" s="3" t="n">
-        <v>2.05</v>
+        <v>1</v>
       </c>
       <c r="AN11" s="2">
         <f>AL11*AM11</f>
         <v/>
       </c>
       <c r="AO11" s="2" t="n"/>
-      <c r="AP11" s="2" t="n"/>
+      <c r="AP11" s="2" t="n">
+        <v>1000</v>
+      </c>
       <c r="AQ11" s="2">
         <f>AN11+N(AO11)+N(AP11)</f>
         <v/>
@@ -7189,552 +7174,8 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>h048</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Krotas</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>1325</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" t="n">
-        <v>851</v>
-      </c>
-      <c r="G12" t="n">
-        <v>858</v>
-      </c>
-      <c r="H12" t="n">
-        <v>854.5</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="J12" t="n">
-        <v>2589.4</v>
-      </c>
-      <c r="K12" t="n">
-        <v>1500</v>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>chaos</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>missile</t>
-        </is>
-      </c>
-      <c r="N12" t="n">
-        <v>850</v>
-      </c>
-      <c r="O12" t="n">
-        <v>1</v>
-      </c>
-      <c r="P12" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>chaos</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>hhou</t>
-        </is>
-      </c>
-      <c r="AE12" s="2" t="n">
-        <v>2500</v>
-      </c>
-      <c r="AF12" t="inlineStr">
-        <is>
-          <t>ANcl,A004,A02X,A014,A028</t>
-        </is>
-      </c>
-      <c r="AG12" t="inlineStr">
-        <is>
-          <t>Up g rade to Krotas - 1325</t>
-        </is>
-      </c>
-      <c r="AK12" t="inlineStr">
-        <is>
-          <t>Activate / Deactivate Mana Detection (ANcl); Versatile Critical Strike I (A004); Gooify (A02X); Combustion (A014); Sell Tower (A028)</t>
-        </is>
-      </c>
-      <c r="AL12" s="2" t="n">
-        <v>2589.4</v>
-      </c>
-      <c r="AM12" s="3" t="n">
-        <v>1.52</v>
-      </c>
-      <c r="AN12" s="2">
-        <f>AL12*AM12</f>
-        <v/>
-      </c>
-      <c r="AO12" s="2" t="n"/>
-      <c r="AP12" s="2" t="n"/>
-      <c r="AQ12" s="2">
-        <f>AN12+N(AO12)+N(AP12)</f>
-        <v/>
-      </c>
-      <c r="AR12" s="3">
-        <f>IF(C12=0,"",AQ12/C12)</f>
-        <v/>
-      </c>
-      <c r="AS12" s="3">
-        <f>IF(C12=0,"",AR12*(K12/725))</f>
-        <v/>
-      </c>
-      <c r="AT12" s="3">
-        <f>(K12/725)^2</f>
-        <v/>
-      </c>
-      <c r="AU12" s="3">
-        <f>IF(C12=0,"",AR12*AT12)</f>
-        <v/>
-      </c>
-      <c r="AV12" t="inlineStr">
-        <is>
-          <t>basic attack</t>
-        </is>
-      </c>
-      <c r="AW12" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>h04G</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Reaperspawn</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>50</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="n">
-        <v>287</v>
-      </c>
-      <c r="G13" t="n">
-        <v>287</v>
-      </c>
-      <c r="H13" t="n">
-        <v>287</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="J13" t="n">
-        <v>358.8</v>
-      </c>
-      <c r="K13" t="n">
-        <v>125</v>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>chaos</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="N13" t="n">
-        <v>286</v>
-      </c>
-      <c r="O13" t="n">
-        <v>1</v>
-      </c>
-      <c r="P13" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>chaos</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>hhou</t>
-        </is>
-      </c>
-      <c r="AD13" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE13" s="2" t="n">
-        <v>1500</v>
-      </c>
-      <c r="AF13" t="inlineStr">
-        <is>
-          <t>A006,A028,ACvp</t>
-        </is>
-      </c>
-      <c r="AG13" t="inlineStr">
-        <is>
-          <t>Up g rade to Reaperspawn</t>
-        </is>
-      </c>
-      <c r="AH13" t="inlineStr">
-        <is>
-          <t>tempest</t>
-        </is>
-      </c>
-      <c r="AI13" t="inlineStr">
-        <is>
-          <t>D2</t>
-        </is>
-      </c>
-      <c r="AJ13" t="inlineStr">
-        <is>
-          <t>AIR CRITICAL STRIKE II identified 2026-09-05 (the Royal Family named the tier: 50% x4). CHAOS attack type - the kit's ONLY non-magic tower. In stock WC3 chaos deals full damage to every armour type, i.e. it ignores the matrix entirely; UNVERIFIED for this map. Melee, but DOES hit air when the flyer passes directly above it (owner 2026-09-05) - so it is a positional anti-air, not a blind spot. 23.90 raw dps/gold is among the best recorded, but it is unadjustable for range and demands exact placement under the flight path.</t>
-        </is>
-      </c>
-      <c r="AK13" t="inlineStr">
-        <is>
-          <t>Air Critical Strike II (A006); Sell Tower (A028); Vampiric Aura (ACvp)</t>
-        </is>
-      </c>
-      <c r="AL13" s="2" t="n">
-        <v>358.8</v>
-      </c>
-      <c r="AM13" s="3" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="AN13" s="2">
-        <f>AL13*AM13</f>
-        <v/>
-      </c>
-      <c r="AO13" s="2" t="n"/>
-      <c r="AP13" s="2" t="n"/>
-      <c r="AQ13" s="2">
-        <f>AN13+N(AO13)+N(AP13)</f>
-        <v/>
-      </c>
-      <c r="AR13" s="3">
-        <f>IF(C13=0,"",AQ13/C13)</f>
-        <v/>
-      </c>
-      <c r="AS13" s="3">
-        <f>IF(C13=0,"",AR13*(K13/725))</f>
-        <v/>
-      </c>
-      <c r="AT13" s="3">
-        <f>(K13/725)^2</f>
-        <v/>
-      </c>
-      <c r="AU13" s="3">
-        <f>IF(C13=0,"",AR13*AT13)</f>
-        <v/>
-      </c>
-      <c r="AV13" t="inlineStr">
-        <is>
-          <t>basic attack</t>
-        </is>
-      </c>
-      <c r="AW13" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>h017</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Sewage Surprise</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>105</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="n">
-        <v>246</v>
-      </c>
-      <c r="G14" t="n">
-        <v>246</v>
-      </c>
-      <c r="H14" t="n">
-        <v>246</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="J14" t="n">
-        <v>289.4</v>
-      </c>
-      <c r="K14" t="n">
-        <v>800</v>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>magic</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>msplash</t>
-        </is>
-      </c>
-      <c r="N14" t="n">
-        <v>245</v>
-      </c>
-      <c r="O14" t="n">
-        <v>1</v>
-      </c>
-      <c r="P14" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>magic</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>hhou</t>
-        </is>
-      </c>
-      <c r="AD14" t="n">
-        <v>7</v>
-      </c>
-      <c r="AE14" s="2" t="n">
-        <v>1500</v>
-      </c>
-      <c r="AF14" t="inlineStr">
-        <is>
-          <t>A03Y,A021,A028,Afra</t>
-        </is>
-      </c>
-      <c r="AG14" t="inlineStr">
-        <is>
-          <t>U pgrade to Sewage Surprise</t>
-        </is>
-      </c>
-      <c r="AH14" t="inlineStr">
-        <is>
-          <t>specialist</t>
-        </is>
-      </c>
-      <c r="AI14" t="inlineStr">
-        <is>
-          <t>D2</t>
-        </is>
-      </c>
-      <c r="AJ14" t="inlineStr">
-        <is>
-          <t>MAGIC (owner 2026-09-06), where its BASE Sewer Barge is siege - so attack type is NOT inherited on upgrade. Consequence: the upgrade gains everywhere except FORTIFIED, where siege 160% vs magic 75% leaves the base nearly as strong as its own upgrade (8.10 vs 5.92). Upgrading is a downgrade on 1 wave in 5. THE AIR BRANCH: this is the T2 upgrade that leads to Interceptor and Arcadia. Choosing the other branch (Brahma Fix It Shop) forfeits the treant's only passive air answer on that Sewer Barge. 'crit mecha like base' - the anti-mecha crit carries.</t>
-        </is>
-      </c>
-      <c r="AK14" t="inlineStr">
-        <is>
-          <t>Machine Critical Strike (A03Y); Splash (A021); Sell Tower (A028); Frost I (Afra)</t>
-        </is>
-      </c>
-      <c r="AL14" s="2" t="n">
-        <v>289.4</v>
-      </c>
-      <c r="AM14" s="3" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="AN14" s="2">
-        <f>AL14*AM14</f>
-        <v/>
-      </c>
-      <c r="AO14" s="2" t="n"/>
-      <c r="AP14" s="2" t="n"/>
-      <c r="AQ14" s="2">
-        <f>AN14+N(AO14)+N(AP14)</f>
-        <v/>
-      </c>
-      <c r="AR14" s="3">
-        <f>IF(C14=0,"",AQ14/C14)</f>
-        <v/>
-      </c>
-      <c r="AS14" s="3">
-        <f>IF(C14=0,"",AR14*(K14/725))</f>
-        <v/>
-      </c>
-      <c r="AT14" s="3">
-        <f>(K14/725)^2</f>
-        <v/>
-      </c>
-      <c r="AU14" s="3">
-        <f>IF(C14=0,"",AR14*AT14)</f>
-        <v/>
-      </c>
-      <c r="AV14" t="inlineStr">
-        <is>
-          <t>basic attack</t>
-        </is>
-      </c>
-      <c r="AW14" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>h047</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Von Chillspeak</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>1225</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" t="n">
-        <v>12000</v>
-      </c>
-      <c r="G15" t="n">
-        <v>12000</v>
-      </c>
-      <c r="H15" t="n">
-        <v>12000</v>
-      </c>
-      <c r="I15" t="n">
-        <v>2</v>
-      </c>
-      <c r="J15" t="n">
-        <v>6000</v>
-      </c>
-      <c r="K15" t="n">
-        <v>1150</v>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>chaos</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>missile</t>
-        </is>
-      </c>
-      <c r="N15" t="n">
-        <v>11999</v>
-      </c>
-      <c r="O15" t="n">
-        <v>1</v>
-      </c>
-      <c r="P15" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>chaos</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>hhou</t>
-        </is>
-      </c>
-      <c r="AE15" s="2" t="n">
-        <v>2500</v>
-      </c>
-      <c r="AF15" t="inlineStr">
-        <is>
-          <t>ANcl,Afrz,Aap1,AIm2,A028</t>
-        </is>
-      </c>
-      <c r="AG15" t="inlineStr">
-        <is>
-          <t>U pgrade to Von Chillspeak - 1225</t>
-        </is>
-      </c>
-      <c r="AK15" t="inlineStr">
-        <is>
-          <t>Activate / Deactivate Mana Detection (ANcl); Stone Cold (Afrz); Grounding Curse (Aap1); Cold Snap (AIm2); Sell Tower (A028)</t>
-        </is>
-      </c>
-      <c r="AL15" s="2" t="n">
-        <v>6000</v>
-      </c>
-      <c r="AM15" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN15" s="2">
-        <f>AL15*AM15</f>
-        <v/>
-      </c>
-      <c r="AO15" s="2" t="n"/>
-      <c r="AP15" s="2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="AQ15" s="2">
-        <f>AN15+N(AO15)+N(AP15)</f>
-        <v/>
-      </c>
-      <c r="AR15" s="3">
-        <f>IF(C15=0,"",AQ15/C15)</f>
-        <v/>
-      </c>
-      <c r="AS15" s="3">
-        <f>IF(C15=0,"",AR15*(K15/725))</f>
-        <v/>
-      </c>
-      <c r="AT15" s="3">
-        <f>(K15/725)^2</f>
-        <v/>
-      </c>
-      <c r="AU15" s="3">
-        <f>IF(C15=0,"",AR15*AT15)</f>
-        <v/>
-      </c>
-      <c r="AV15" t="inlineStr">
-        <is>
-          <t>basic attack</t>
-        </is>
-      </c>
-      <c r="AW15" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:AW15"/>
+  <autoFilter ref="A1:AW11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17624,10 +17065,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA23"/>
+  <dimension ref="A1:BA22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
@@ -17662,7 +17103,7 @@
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="11" customWidth="1" min="34" max="34"/>
     <col width="26" customWidth="1" min="35" max="35"/>
-    <col width="33" customWidth="1" min="36" max="36"/>
+    <col width="35" customWidth="1" min="36" max="36"/>
     <col width="11" customWidth="1" min="37" max="37"/>
     <col width="46" customWidth="1" min="38" max="38"/>
     <col width="17" customWidth="1" min="39" max="39"/>
@@ -17679,7 +17120,7 @@
     <col width="22" customWidth="1" min="50" max="50"/>
     <col width="48" customWidth="1" min="51" max="51"/>
     <col width="13" customWidth="1" min="52" max="52"/>
-    <col width="19" customWidth="1" min="53" max="53"/>
+    <col width="20" customWidth="1" min="53" max="53"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -20930,7 +20371,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Sewage Surprise</t>
+          <t>Specialist Base</t>
         </is>
       </c>
       <c r="AA21" s="2" t="n"/>
@@ -20939,14 +20380,9 @@
           <t>hand capture only — no extracted counterpart</t>
         </is>
       </c>
-      <c r="AM21" t="inlineStr">
-        <is>
-          <t>D2</t>
-        </is>
-      </c>
       <c r="AN21" t="inlineStr">
         <is>
-          <t>MAGIC (owner 2026-09-06), where its BASE Sewer Barge is siege - so attack type is NOT inherited on upgrade. Consequence: the upgrade gains everywhere except FORTIFIED, where siege 160% vs magic 75% leaves the base nearly as strong as its own upgrade (8.10 vs 5.92). Upgrading is a downgrade on 1 wave in 5. THE AIR BRANCH: this is the T2 upgrade that leads to Interceptor and Arcadia. Choosing the other branch (Brahma Fix It Shop) forfeits the treant's only passive air answer on that Sewer Barge. 'crit mecha like base' - the anti-mecha crit carries.</t>
+          <t>THE TREANT HAS A BASE UPGRADE TOO. Analogous to the Royal Family's Royal Base II, which is bought at the hero-selection building. So base upgrades are present in 2 of 3 captured kits - the Tempest Hawk, which has none, is the exception. Cost and purchase location unread.</t>
         </is>
       </c>
       <c r="AO21" s="2" t="n"/>
@@ -20988,13 +20424,91 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Brahma Fix It Shop</t>
-        </is>
-      </c>
-      <c r="AA22" s="2" t="n"/>
+          <t>Brahma's Fix-it Shop</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>h04H</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>95</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Machine Critical Strike (A03Y); Super Regeneration (A070); Empathic Fix (AChv); Sell Tower (A028)</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>175</v>
+      </c>
+      <c r="K22" t="n">
+        <v>175</v>
+      </c>
+      <c r="L22" t="n">
+        <v>175</v>
+      </c>
+      <c r="M22" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N22" t="n">
+        <v>1100</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>siege</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>116.7</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>7</v>
+      </c>
+      <c r="AA22" s="2" t="n">
+        <v>1500</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>missile</t>
+        </is>
+      </c>
+      <c r="AD22" t="n">
+        <v>174</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>siege</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr">
+        <is>
+          <t>hhou</t>
+        </is>
+      </c>
+      <c r="AI22" t="inlineStr">
+        <is>
+          <t>A03Y,A070,AChv,A028</t>
+        </is>
+      </c>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>Up g rade to Brahma's Fix-it Shop</t>
+        </is>
+      </c>
       <c r="AL22" t="inlineStr">
         <is>
-          <t>hand capture only — no extracted counterpart</t>
+          <t>relocated</t>
         </is>
       </c>
       <c r="AM22" t="inlineStr">
@@ -21007,9 +20521,11 @@
           <t>SIEGE (owner 2026-09-06) - and that sharpens the T2 fork: the air branch (Sewage Surprise) switches the line to MAGIC, while this branch KEEPS siege. So the fork is siege-stays vs magic-switch, not two arbitrary paths. Its 4.67 becomes 7.47 on Fortified. THE GENERALIST BRANCH: leads to Little Jack and Battleship Mackinaw (22.07 untyped, the kit's best all-purpose tower). The opposite branch leads to the air line. Support branch. Longest range in the captured kit (1100). 'same passive to crit unit' - target type not stated.</t>
         </is>
       </c>
-      <c r="AO22" s="2" t="n"/>
+      <c r="AO22" s="2" t="n">
+        <v>116.7</v>
+      </c>
       <c r="AP22" s="3" t="n">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="AQ22" s="2">
         <f>AO22*AP22</f>
@@ -21039,65 +20555,22 @@
       </c>
       <c r="AY22" t="inlineStr">
         <is>
-          <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Specialist Base</t>
-        </is>
-      </c>
-      <c r="AA23" s="2" t="n"/>
-      <c r="AL23" t="inlineStr">
-        <is>
-          <t>hand capture only — no extracted counterpart</t>
-        </is>
-      </c>
-      <c r="AN23" t="inlineStr">
-        <is>
-          <t>THE TREANT HAS A BASE UPGRADE TOO. Analogous to the Royal Family's Royal Base II, which is bought at the hero-selection building. So base upgrades are present in 2 of 3 captured kits - the Tempest Hawk, which has none, is the exception. Cost and purchase location unread.</t>
-        </is>
-      </c>
-      <c r="AO23" s="2" t="n"/>
-      <c r="AP23" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ23" s="2">
-        <f>AO23*AP23</f>
-        <v/>
-      </c>
-      <c r="AR23" s="3">
-        <f>IF(D23=0,"",AW23/D23)</f>
-        <v/>
-      </c>
-      <c r="AS23" s="3">
-        <f>(N23/725)^2</f>
-        <v/>
-      </c>
-      <c r="AT23" s="3">
-        <f>IF(D23=0,"",AR23*AS23)</f>
-        <v/>
-      </c>
-      <c r="AU23" s="2" t="n"/>
-      <c r="AV23" s="2" t="n"/>
-      <c r="AW23" s="2">
-        <f>AQ23+N(AU23)+N(AV23)</f>
-        <v/>
-      </c>
-      <c r="AX23" s="3">
-        <f>IF(D23=0,"",AR23*(N23/725))</f>
-        <v/>
-      </c>
-      <c r="AY23" t="inlineStr">
-        <is>
-          <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
+          <t>basic attack</t>
+        </is>
+      </c>
+      <c r="AZ22" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="BA22" t="inlineStr">
+        <is>
+          <t>Brahma Fix It Shop</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BA23"/>
+  <autoFilter ref="A1:BA22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21108,7 +20581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB22"/>
+  <dimension ref="A1:BB21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -21150,7 +20623,7 @@
     <col width="11" customWidth="1" min="37" max="37"/>
     <col width="11" customWidth="1" min="38" max="38"/>
     <col width="12" customWidth="1" min="39" max="39"/>
-    <col width="46" customWidth="1" min="40" max="40"/>
+    <col width="11" customWidth="1" min="40" max="40"/>
     <col width="17" customWidth="1" min="41" max="41"/>
     <col width="48" customWidth="1" min="42" max="42"/>
     <col width="9" customWidth="1" min="43" max="43"/>
@@ -24418,13 +23891,91 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Father Dragon</t>
-        </is>
-      </c>
-      <c r="AA21" s="2" t="n"/>
+          <t>Reaperspawn</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>h04G</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>50</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Air Critical Strike II (A006); Sell Tower (A028); Vampiric Aura (ACvp)</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>287</v>
+      </c>
+      <c r="K21" t="n">
+        <v>287</v>
+      </c>
+      <c r="L21" t="n">
+        <v>287</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="N21" t="n">
+        <v>125</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>chaos</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>358.8</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA21" s="2" t="n">
+        <v>1500</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="AD21" t="n">
+        <v>286</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>chaos</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr">
+        <is>
+          <t>hhou</t>
+        </is>
+      </c>
+      <c r="AI21" t="inlineStr">
+        <is>
+          <t>A006,A028,ACvp</t>
+        </is>
+      </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>Up g rade to Reaperspawn</t>
+        </is>
+      </c>
       <c r="AN21" t="inlineStr">
         <is>
-          <t>hand capture only — no extracted counterpart</t>
+          <t>relocated</t>
         </is>
       </c>
       <c r="AO21" t="inlineStr">
@@ -24434,12 +23985,14 @@
       </c>
       <c r="AP21" t="inlineStr">
         <is>
-          <t xml:space="preserve">AIR CRITICAL STRIKE II identified 2026-09-05 (the Royal Family named the tier: 50% x4). RESOLVED 2026-09-05: the trait is named "Boss Assassin" but TARGETS HEROES - the owner read "boss assassin II (50% x8 against heroes)" on a Royal Family tower. So the earlier boss-vs-hero ambiguity was the GAME conflating them, not a transcription slip. Both readings were right. DUAL crit (air AND boss) at 50% x4 each. 16.78 range-adjusted against either. Its 600 range is short for the kit. </t>
-        </is>
-      </c>
-      <c r="AQ21" s="2" t="n"/>
+          <t>AIR CRITICAL STRIKE II identified 2026-09-05 (the Royal Family named the tier: 50% x4). CHAOS attack type - the kit's ONLY non-magic tower. In stock WC3 chaos deals full damage to every armour type, i.e. it ignores the matrix entirely; UNVERIFIED for this map. Melee, but DOES hit air when the flyer passes directly above it (owner 2026-09-05) - so it is a positional anti-air, not a blind spot. 23.90 raw dps/gold is among the best recorded, but it is unadjustable for range and demands exact placement under the flight path.</t>
+        </is>
+      </c>
+      <c r="AQ21" s="2" t="n">
+        <v>358.8</v>
+      </c>
       <c r="AR21" s="3" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="AS21" s="2">
         <f>AQ21*AR21</f>
@@ -24469,70 +24022,17 @@
       </c>
       <c r="BA21" t="inlineStr">
         <is>
-          <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Reaper Spawn</t>
-        </is>
-      </c>
-      <c r="AA22" s="2" t="n"/>
-      <c r="AN22" t="inlineStr">
-        <is>
-          <t>hand capture only — no extracted counterpart</t>
-        </is>
-      </c>
-      <c r="AO22" t="inlineStr">
-        <is>
-          <t>D2</t>
-        </is>
-      </c>
-      <c r="AP22" t="inlineStr">
-        <is>
-          <t>AIR CRITICAL STRIKE II identified 2026-09-05 (the Royal Family named the tier: 50% x4). CHAOS attack type - the kit's ONLY non-magic tower. In stock WC3 chaos deals full damage to every armour type, i.e. it ignores the matrix entirely; UNVERIFIED for this map. Melee, but DOES hit air when the flyer passes directly above it (owner 2026-09-05) - so it is a positional anti-air, not a blind spot. 23.90 raw dps/gold is among the best recorded, but it is unadjustable for range and demands exact placement under the flight path.</t>
-        </is>
-      </c>
-      <c r="AQ22" s="2" t="n"/>
-      <c r="AR22" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS22" s="2">
-        <f>AQ22*AR22</f>
-        <v/>
-      </c>
-      <c r="AT22" s="3">
-        <f>IF(D22=0,"",AY22/D22)</f>
-        <v/>
-      </c>
-      <c r="AU22" s="3">
-        <f>(N22/725)^2</f>
-        <v/>
-      </c>
-      <c r="AV22" s="3">
-        <f>IF(D22=0,"",AT22*AU22)</f>
-        <v/>
-      </c>
-      <c r="AW22" s="2" t="n"/>
-      <c r="AX22" s="2" t="n"/>
-      <c r="AY22" s="2">
-        <f>AS22+N(AW22)+N(AX22)</f>
-        <v/>
-      </c>
-      <c r="AZ22" s="3">
-        <f>IF(D22=0,"",AT22*(N22/725))</f>
-        <v/>
-      </c>
-      <c r="BA22" t="inlineStr">
-        <is>
-          <t>no damage figure — support/on-death, or a bonus that needs a basic attack it lacks</t>
+          <t>basic attack</t>
+        </is>
+      </c>
+      <c r="BB21" t="inlineStr">
+        <is>
+          <t>map</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BB22"/>
+  <autoFilter ref="A1:BB21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24806,11 +24306,11 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Tamed Game; Toxic Assassin; Father Dragon</t>
+          <t>Tamed Game; Toxic Assassin; Frigid Dryad</t>
         </is>
       </c>
     </row>
@@ -24871,11 +24371,11 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Axeman; Ruthless Warlord; Father Dragon</t>
+          <t>Axeman; Ruthless Warlord; Jailing Officer</t>
         </is>
       </c>
     </row>
@@ -25771,11 +25271,11 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Orobos Slave; Sewage Surprise; Frigid Dryad</t>
+          <t>Orobos Slave; Frigid Dryad; Iron Mistress</t>
         </is>
       </c>
     </row>
@@ -25861,11 +25361,11 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Brahma's Fix-it Shop; Equipped Peasant 1; Equipped Peasant 2</t>
+          <t>Equipped Peasant 1; Equipped Peasant 2; Equipped Peasant 3</t>
         </is>
       </c>
     </row>
@@ -26071,11 +25571,11 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Myrkridon Trow; Father Dragon; Hunter</t>
+          <t>Myrkridon Trow; Hunter; Jailing Officer</t>
         </is>
       </c>
     </row>
@@ -26401,11 +25901,11 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Brahma's Fix-it Shop; Sewage Surprise; Xavier</t>
+          <t>Xavier; Sewer Barge; Frankenstone</t>
         </is>
       </c>
     </row>
@@ -27096,7 +26596,7 @@
         </is>
       </c>
       <c r="G84" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
@@ -40653,37 +40153,37 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>tempest</t>
+          <t>arcane</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="C5" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D5" t="n">
-        <v>4.2</v>
+        <v>2.04</v>
       </c>
       <c r="E5" t="n">
-        <v>850</v>
+        <v>1150</v>
       </c>
       <c r="F5" t="n">
-        <v>5.84</v>
+        <v>5.43</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Jenovaroth</t>
+          <t>Fire Hydra</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>800</v>
+        <v>255</v>
       </c>
       <c r="I5" t="n">
-        <v>101.25</v>
+        <v>6.41</v>
       </c>
       <c r="J5" t="n">
-        <v>21722</v>
+        <v>1357</v>
       </c>
       <c r="K5" t="n">
         <v>5</v>
@@ -40692,37 +40192,37 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>arcane</t>
+          <t>tempest</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="C6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D6" t="n">
-        <v>2.04</v>
+        <v>4.24</v>
       </c>
       <c r="E6" t="n">
-        <v>1150</v>
+        <v>800</v>
       </c>
       <c r="F6" t="n">
-        <v>5.43</v>
+        <v>5.22</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Fire Hydra</t>
+          <t>Jenovaroth</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>255</v>
+        <v>800</v>
       </c>
       <c r="I6" t="n">
-        <v>6.41</v>
+        <v>101.25</v>
       </c>
       <c r="J6" t="n">
-        <v>1357</v>
+        <v>21722</v>
       </c>
       <c r="K6" t="n">
         <v>5</v>
@@ -40735,16 +40235,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C7" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D7" t="n">
-        <v>4.41</v>
+        <v>4.35</v>
       </c>
       <c r="E7" t="n">
-        <v>800</v>
+        <v>850</v>
       </c>
       <c r="F7" t="n">
         <v>5.09</v>

</xml_diff>

<commit_message>
Targeting now reads BOTH weapons — seven towers were misdescribed
The targets column held only attack 1. Seven towers have a second enabled attack
(uaen=3) covering what the first does not, so all seven hit air AND ground —
Jenovaroth read as air-only, six others as ground-only. New hits_air / hits_ground /
targets_all / attack_count columns computed from the union of enabled weapons.
</commit_message>
<xml_diff>
--- a/skibi-data.xlsx
+++ b/skibi-data.xlsx
@@ -30,23 +30,23 @@
     <sheet name="waves" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'arcane'!$A$1:$AV$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'arcane'!$A$1:$AZ$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'armour_matrix'!$A$1:$F$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'bosses'!$A$1:$O$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'caster_dps'!$A$1:$L$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'game_modes'!$A$1:$I$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'hero_ranking'!$A$1:$K$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'heroes'!$A$1:$H$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'military'!$A$1:$AY$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'military'!$A$1:$BC$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'minigame_items'!$A$1:$D$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'minigame_readings'!$A$1:$G$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'minigames'!$A$1:$I$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'other_towers'!$A$1:$AW$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'ranger'!$A$1:$AV$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'royal_family'!$A$1:$BC$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'scarlet_knight'!$A$1:$AV$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'specialist'!$A$1:$BA$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'tempest'!$A$1:$BB$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'ranger'!$A$1:$AZ$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'royal_family'!$A$1:$BG$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'scarlet_knight'!$A$1:$AZ$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'specialist'!$A$1:$BE$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'tempest'!$A$1:$BF$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'tower_traits'!$A$1:$I$113</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'wave_modifiers'!$A$1:$D$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'wave_traits'!$A$1:$K$51</definedName>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV18"/>
+  <dimension ref="A1:AZ18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -514,6 +514,10 @@
     <col width="22" customWidth="1" min="46" max="46"/>
     <col width="48" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
+    <col width="14" customWidth="1" min="49" max="49"/>
+    <col width="10" customWidth="1" min="50" max="50"/>
+    <col width="13" customWidth="1" min="51" max="51"/>
+    <col width="31" customWidth="1" min="52" max="52"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -757,6 +761,26 @@
           <t>cost_source</t>
         </is>
       </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>attack_count</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>hits_air</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>hits_ground</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>targets_all</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -839,6 +863,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -923,6 +965,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1005,6 +1065,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1089,6 +1167,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1173,6 +1269,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1255,6 +1369,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1411,6 +1543,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1493,6 +1643,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ10" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1637,6 +1805,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ11" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1781,6 +1967,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ12" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1865,6 +2069,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ13" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1949,6 +2171,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ14" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2228,7 +2468,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AV18"/>
+  <autoFilter ref="A1:AZ18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7186,7 +7426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV20"/>
+  <dimension ref="A1:AZ20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7237,6 +7477,10 @@
     <col width="22" customWidth="1" min="46" max="46"/>
     <col width="14" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
+    <col width="14" customWidth="1" min="49" max="49"/>
+    <col width="10" customWidth="1" min="50" max="50"/>
+    <col width="13" customWidth="1" min="51" max="51"/>
+    <col width="31" customWidth="1" min="52" max="52"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7480,6 +7724,26 @@
           <t>cost_source</t>
         </is>
       </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>attack_count</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>hits_air</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>hits_ground</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>targets_all</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7624,6 +7888,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7768,6 +8050,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7917,6 +8217,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8063,6 +8381,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8209,6 +8545,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8353,6 +8707,24 @@
       <c r="AV7" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="AW7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -8499,6 +8871,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -8638,6 +9028,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8787,6 +9195,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ10" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -8936,6 +9362,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ11" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9080,6 +9524,24 @@
       <c r="AV12" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="AW12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ12" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -9231,6 +9693,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ13" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9375,6 +9855,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ14" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -9519,6 +10017,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ15" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9665,6 +10181,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ16" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9811,6 +10345,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ17" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9957,6 +10509,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ18" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -10098,6 +10668,24 @@
       <c r="AV19" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="AW19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ19" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -10249,9 +10837,27 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ20" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AV20"/>
+  <autoFilter ref="A1:AZ20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10262,7 +10868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC23"/>
+  <dimension ref="A1:BG23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -10320,6 +10926,10 @@
     <col width="48" customWidth="1" min="53" max="53"/>
     <col width="13" customWidth="1" min="54" max="54"/>
     <col width="21" customWidth="1" min="55" max="55"/>
+    <col width="14" customWidth="1" min="56" max="56"/>
+    <col width="10" customWidth="1" min="57" max="57"/>
+    <col width="13" customWidth="1" min="58" max="58"/>
+    <col width="31" customWidth="1" min="59" max="59"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10598,6 +11208,26 @@
           <t>hand_capture_name</t>
         </is>
       </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>attack_count</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>hits_air</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>hits_ground</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>targets_all</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -10757,6 +11387,24 @@
           <t>Grayson Fort Buster</t>
         </is>
       </c>
+      <c r="BD2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG2" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -10911,6 +11559,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BD3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG3" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -11030,6 +11696,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BD4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG4" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -11196,6 +11880,24 @@
       <c r="BC5" t="inlineStr">
         <is>
           <t>Tyr Spirit</t>
+        </is>
+      </c>
+      <c r="BD5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG5" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -11357,6 +12059,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BD6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG6" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -11513,6 +12233,24 @@
       <c r="BC7" t="inlineStr">
         <is>
           <t>Peepy Bronzebeard</t>
+        </is>
+      </c>
+      <c r="BD7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG7" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -11701,6 +12439,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BD8" t="n">
+        <v>2</v>
+      </c>
+      <c r="BE8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG8" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -11855,6 +12611,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BD9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG9" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12014,6 +12788,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BD10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG10" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -12170,6 +12962,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BD11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG11" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -12324,6 +13134,24 @@
       <c r="BB12" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="BD12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG12" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -12490,6 +13318,24 @@
           <t>Petrified Shell</t>
         </is>
       </c>
+      <c r="BD13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG13" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -12644,6 +13490,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BD14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG14" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -12803,6 +13667,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BD15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG15" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -12962,6 +13844,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BD16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG16" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -13111,6 +14011,24 @@
       <c r="BB17" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="BD17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG17" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -13262,6 +14180,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BD18" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG18" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -13408,6 +14344,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BD19" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG19" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -13557,6 +14511,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BD20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG20" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -13716,6 +14688,24 @@
           <t>Lilliana May</t>
         </is>
       </c>
+      <c r="BD21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG21" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -13897,6 +14887,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BD22" t="n">
+        <v>2</v>
+      </c>
+      <c r="BE22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG22" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -13952,7 +14960,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BC23"/>
+  <autoFilter ref="A1:BG23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13963,7 +14971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV21"/>
+  <dimension ref="A1:AZ21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -14014,6 +15022,10 @@
     <col width="22" customWidth="1" min="46" max="46"/>
     <col width="48" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
+    <col width="14" customWidth="1" min="49" max="49"/>
+    <col width="10" customWidth="1" min="50" max="50"/>
+    <col width="13" customWidth="1" min="51" max="51"/>
+    <col width="31" customWidth="1" min="52" max="52"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14257,6 +15269,26 @@
           <t>cost_source</t>
         </is>
       </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>attack_count</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>hits_air</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>hits_ground</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>targets_all</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -14396,6 +15428,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -14535,6 +15585,24 @@
       <c r="AV3" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="AW3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -14686,6 +15754,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -14775,6 +15861,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -14924,6 +16028,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -15073,6 +16195,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -15212,6 +16352,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -15356,6 +16514,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -15505,6 +16681,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ10" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -15654,6 +16848,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ11" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -15743,6 +16955,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ12" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -15887,6 +17117,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ13" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -16033,6 +17281,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ14" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -16179,6 +17445,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ15" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -16328,6 +17612,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ16" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -16477,6 +17779,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ17" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -16621,6 +17941,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ18" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -16762,6 +18100,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ19" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -16906,6 +18262,24 @@
       <c r="AV20" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="AW20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ20" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -17052,9 +18426,27 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AW21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ21" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AV21"/>
+  <autoFilter ref="A1:AZ21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17065,7 +18457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA22"/>
+  <dimension ref="A1:BE22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17121,6 +18513,10 @@
     <col width="48" customWidth="1" min="51" max="51"/>
     <col width="13" customWidth="1" min="52" max="52"/>
     <col width="20" customWidth="1" min="53" max="53"/>
+    <col width="14" customWidth="1" min="54" max="54"/>
+    <col width="10" customWidth="1" min="55" max="55"/>
+    <col width="13" customWidth="1" min="56" max="56"/>
+    <col width="31" customWidth="1" min="57" max="57"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -17389,6 +18785,26 @@
           <t>hand_capture_name</t>
         </is>
       </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>attack_count</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>hits_air</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>hits_ground</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>targets_all</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -17548,6 +18964,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BB2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE2" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -17707,6 +19141,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BB3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE3" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -17863,6 +19315,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BB4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE4" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -18029,6 +19499,24 @@
           <t>Giga Spikes</t>
         </is>
       </c>
+      <c r="BB5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE5" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -18182,6 +19670,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BB6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE6" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -18333,6 +19839,24 @@
       <c r="AZ7" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="BB7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE7" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -18481,6 +20005,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BB8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE8" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -18630,6 +20172,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BB9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE9" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -18789,6 +20349,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BB10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE10" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -18948,6 +20526,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BB11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE11" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -19102,6 +20698,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BB12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE12" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -19258,6 +20872,24 @@
       <c r="AZ13" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="BB13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE13" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -19428,6 +21060,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BB14" t="n">
+        <v>2</v>
+      </c>
+      <c r="BC14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE14" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -19587,6 +21237,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BB15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE15" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -19746,6 +21414,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BB16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE16" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -19905,6 +21591,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BB17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE17" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -20059,6 +21763,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BB18" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE18" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -20218,6 +21940,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BB19" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE19" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -20367,6 +22107,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BB20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE20" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -20568,9 +22326,27 @@
           <t>Brahma Fix It Shop</t>
         </is>
       </c>
+      <c r="BB22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE22" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BA22"/>
+  <autoFilter ref="A1:BE22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20581,7 +22357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB21"/>
+  <dimension ref="A1:BF21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -20638,6 +22414,10 @@
     <col width="22" customWidth="1" min="52" max="52"/>
     <col width="48" customWidth="1" min="53" max="53"/>
     <col width="13" customWidth="1" min="54" max="54"/>
+    <col width="14" customWidth="1" min="55" max="55"/>
+    <col width="10" customWidth="1" min="56" max="56"/>
+    <col width="13" customWidth="1" min="57" max="57"/>
+    <col width="31" customWidth="1" min="58" max="58"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -20911,6 +22691,26 @@
           <t>cost_source</t>
         </is>
       </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>attack_count</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>hits_air</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>hits_ground</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>targets_all</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -21070,6 +22870,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF2" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -21224,6 +23042,24 @@
       <c r="BB3" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="BC3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF3" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -21385,6 +23221,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF4" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -21544,6 +23398,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF5" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -21698,6 +23570,24 @@
       <c r="BB6" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="BC6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF6" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -21854,6 +23744,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF7" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -22008,6 +23916,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF8" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -22162,6 +24088,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF9" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -22321,6 +24265,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF10" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -22506,6 +24468,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC11" t="n">
+        <v>2</v>
+      </c>
+      <c r="BD11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF11" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -22662,6 +24642,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF12" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -22816,6 +24814,24 @@
       <c r="BB13" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="BC13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF13" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -22972,6 +24988,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF14" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -23128,6 +25162,24 @@
       <c r="BB15" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="BC15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF15" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -23224,6 +25276,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF16" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -23378,6 +25448,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF17" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -23564,6 +25652,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC18" t="n">
+        <v>2</v>
+      </c>
+      <c r="BD18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF18" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -23715,6 +25821,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC19" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF19" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -23885,6 +26009,24 @@
       <c r="BB20" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="BC20" t="n">
+        <v>2</v>
+      </c>
+      <c r="BD20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF20" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -24030,9 +26172,27 @@
           <t>map</t>
         </is>
       </c>
+      <c r="BC21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF21" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BB21"/>
+  <autoFilter ref="A1:BF21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -41715,7 +43875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY20"/>
+  <dimension ref="A1:BC20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -41769,6 +43929,10 @@
     <col width="22" customWidth="1" min="49" max="49"/>
     <col width="14" customWidth="1" min="50" max="50"/>
     <col width="13" customWidth="1" min="51" max="51"/>
+    <col width="14" customWidth="1" min="52" max="52"/>
+    <col width="10" customWidth="1" min="53" max="53"/>
+    <col width="13" customWidth="1" min="54" max="54"/>
+    <col width="31" customWidth="1" min="55" max="55"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -42027,6 +44191,26 @@
           <t>cost_source</t>
         </is>
       </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>attack_count</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>hits_air</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>hits_ground</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>targets_all</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -42166,6 +44350,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AZ2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -42305,6 +44507,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AZ3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC3" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -42446,6 +44666,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AZ4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC4" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -42585,6 +44823,24 @@
       <c r="AY5" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="AZ5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC5" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -42731,6 +44987,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AZ6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC6" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -42880,6 +45154,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AZ7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC7" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -43014,6 +45306,24 @@
       <c r="AY8" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="AZ8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC8" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -43150,6 +45460,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AZ9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC9" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -43294,6 +45622,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AZ10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC10" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -43438,6 +45784,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AZ11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC11" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -43577,6 +45941,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AZ12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC12" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -43713,6 +46095,24 @@
       <c r="AY13" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="AZ13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC13" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -43849,6 +46249,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AZ14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC14" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -43990,6 +46408,24 @@
       <c r="AY15" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="AZ15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC15" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -44143,6 +46579,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AZ16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC16" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -44284,6 +46738,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AZ17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC17" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -44455,6 +46927,24 @@
       <c r="AY18" t="inlineStr">
         <is>
           <t>map</t>
+        </is>
+      </c>
+      <c r="AZ18" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC18" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
     </row>
@@ -44593,6 +47083,24 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AZ19" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC19" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -44732,9 +47240,27 @@
           <t>map</t>
         </is>
       </c>
+      <c r="AZ20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BC20" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AY20"/>
+  <autoFilter ref="A1:BC20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Per-target-type dps (dps_vs_ground / dps_vs_air) for dual-weapon towers
</commit_message>
<xml_diff>
--- a/skibi-data.xlsx
+++ b/skibi-data.xlsx
@@ -30,23 +30,23 @@
     <sheet name="waves" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'arcane'!$A$1:$AZ$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'arcane'!$A$1:$BD$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'armour_matrix'!$A$1:$F$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'bosses'!$A$1:$O$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'caster_dps'!$A$1:$L$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'game_modes'!$A$1:$I$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'hero_ranking'!$A$1:$K$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'heroes'!$A$1:$H$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'military'!$A$1:$BC$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'military'!$A$1:$BG$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'minigame_items'!$A$1:$D$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'minigame_readings'!$A$1:$G$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'minigames'!$A$1:$I$80</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'other_towers'!$A$1:$AW$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'ranger'!$A$1:$AZ$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'royal_family'!$A$1:$BG$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'scarlet_knight'!$A$1:$AZ$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'specialist'!$A$1:$BE$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'tempest'!$A$1:$BF$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'other_towers'!$A$1:$AY$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'ranger'!$A$1:$BD$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'royal_family'!$A$1:$BK$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'scarlet_knight'!$A$1:$BD$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'specialist'!$A$1:$BI$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'tempest'!$A$1:$BJ$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'tower_traits'!$A$1:$I$113</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'wave_modifiers'!$A$1:$D$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'wave_traits'!$A$1:$K$51</definedName>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ18"/>
+  <dimension ref="A1:BD18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -518,6 +518,10 @@
     <col width="10" customWidth="1" min="50" max="50"/>
     <col width="13" customWidth="1" min="51" max="51"/>
     <col width="31" customWidth="1" min="52" max="52"/>
+    <col width="31" customWidth="1" min="53" max="53"/>
+    <col width="14" customWidth="1" min="54" max="54"/>
+    <col width="15" customWidth="1" min="55" max="55"/>
+    <col width="12" customWidth="1" min="56" max="56"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -781,6 +785,26 @@
           <t>targets_all</t>
         </is>
       </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>atk1_targets</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>atk2_targets</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>dps_vs_ground</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>dps_vs_air</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -881,6 +905,11 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -983,6 +1012,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA3" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC3" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="BD3" t="n">
+        <v>39.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1083,6 +1123,11 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA4" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1185,6 +1230,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA5" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC5" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="BD5" t="n">
+        <v>47.3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1287,6 +1343,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA6" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC6" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>48.6</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1387,6 +1454,11 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1561,6 +1633,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC9" t="n">
+        <v>58</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1661,6 +1744,11 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA10" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1823,6 +1911,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA11" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC11" t="n">
+        <v>710</v>
+      </c>
+      <c r="BD11" t="n">
+        <v>710</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1985,6 +2084,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA12" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC12" t="n">
+        <v>649.4</v>
+      </c>
+      <c r="BD12" t="n">
+        <v>649.4</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2087,6 +2197,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA13" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC13" t="n">
+        <v>857.1</v>
+      </c>
+      <c r="BD13" t="n">
+        <v>857.1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2189,6 +2310,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA14" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC14" t="n">
+        <v>1356.7</v>
+      </c>
+      <c r="BD14" t="n">
+        <v>1356.7</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2468,7 +2600,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AZ18"/>
+  <autoFilter ref="A1:BD18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5882,7 +6014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW11"/>
+  <dimension ref="A1:AY11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5934,6 +6066,8 @@
     <col width="27" customWidth="1" min="47" max="47"/>
     <col width="14" customWidth="1" min="48" max="48"/>
     <col width="13" customWidth="1" min="49" max="49"/>
+    <col width="15" customWidth="1" min="50" max="50"/>
+    <col width="12" customWidth="1" min="51" max="51"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6182,6 +6316,16 @@
           <t>cost_source</t>
         </is>
       </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>dps_vs_ground</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>dps_vs_air</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7415,7 +7559,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AW11"/>
+  <autoFilter ref="A1:AY11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7426,7 +7570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ20"/>
+  <dimension ref="A1:BD20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7481,6 +7625,10 @@
     <col width="10" customWidth="1" min="50" max="50"/>
     <col width="13" customWidth="1" min="51" max="51"/>
     <col width="31" customWidth="1" min="52" max="52"/>
+    <col width="31" customWidth="1" min="53" max="53"/>
+    <col width="14" customWidth="1" min="54" max="54"/>
+    <col width="15" customWidth="1" min="55" max="55"/>
+    <col width="12" customWidth="1" min="56" max="56"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7744,6 +7892,26 @@
           <t>targets_all</t>
         </is>
       </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>atk1_targets</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>atk2_targets</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>dps_vs_ground</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>dps_vs_air</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7906,6 +8074,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC2" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>46.8</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8068,6 +8247,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA3" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC3" t="n">
+        <v>345</v>
+      </c>
+      <c r="BD3" t="n">
+        <v>345</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8235,6 +8425,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA4" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC4" t="n">
+        <v>142.5</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>142.5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8399,6 +8600,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA5" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC5" t="n">
+        <v>1252.1</v>
+      </c>
+      <c r="BD5" t="n">
+        <v>1252.1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8563,6 +8775,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA6" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC6" t="n">
+        <v>274</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>274</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8726,6 +8949,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC7" t="n">
+        <v>1007</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>1007</v>
       </c>
     </row>
     <row r="8">
@@ -8889,6 +9123,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC8" t="n">
+        <v>2536.9</v>
+      </c>
+      <c r="BD8" t="n">
+        <v>2536.9</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -9046,6 +9291,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC9" t="n">
+        <v>113</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9213,6 +9469,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA10" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC10" t="n">
+        <v>542.5</v>
+      </c>
+      <c r="BD10" t="n">
+        <v>542.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9380,6 +9647,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA11" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC11" t="n">
+        <v>3362.1</v>
+      </c>
+      <c r="BD11" t="n">
+        <v>3362.1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9543,6 +9821,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BA12" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC12" t="n">
+        <v>322.2</v>
+      </c>
+      <c r="BD12" t="n">
+        <v>322.2</v>
       </c>
     </row>
     <row r="13">
@@ -9711,6 +10000,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA13" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC13" t="n">
+        <v>1064.4</v>
+      </c>
+      <c r="BD13" t="n">
+        <v>1064.4</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9873,6 +10173,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA14" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC14" t="n">
+        <v>975</v>
+      </c>
+      <c r="BD14" t="n">
+        <v>975</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -10035,6 +10346,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA15" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC15" t="n">
+        <v>689.3</v>
+      </c>
+      <c r="BD15" t="n">
+        <v>689.3</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -10199,6 +10521,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA16" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC16" t="n">
+        <v>1883.4</v>
+      </c>
+      <c r="BD16" t="n">
+        <v>1883.4</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -10363,6 +10696,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA17" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC17" t="n">
+        <v>4874.8</v>
+      </c>
+      <c r="BD17" t="n">
+        <v>4874.8</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -10527,6 +10871,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA18" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC18" t="n">
+        <v>14960.4</v>
+      </c>
+      <c r="BD18" t="n">
+        <v>14960.4</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -10687,6 +11042,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BA19" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC19" t="n">
+        <v>4041.3</v>
+      </c>
+      <c r="BD19" t="n">
+        <v>4041.3</v>
       </c>
     </row>
     <row r="20">
@@ -10855,9 +11221,20 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA20" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC20" t="n">
+        <v>6926.1</v>
+      </c>
+      <c r="BD20" t="n">
+        <v>6926.1</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AZ20"/>
+  <autoFilter ref="A1:BD20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10868,7 +11245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG23"/>
+  <dimension ref="A1:BK23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -10930,6 +11307,10 @@
     <col width="10" customWidth="1" min="57" max="57"/>
     <col width="13" customWidth="1" min="58" max="58"/>
     <col width="31" customWidth="1" min="59" max="59"/>
+    <col width="31" customWidth="1" min="60" max="60"/>
+    <col width="24" customWidth="1" min="61" max="61"/>
+    <col width="15" customWidth="1" min="62" max="62"/>
+    <col width="12" customWidth="1" min="63" max="63"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11228,6 +11609,26 @@
           <t>targets_all</t>
         </is>
       </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>atk1_targets</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>atk2_targets</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>dps_vs_ground</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>dps_vs_air</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -11405,6 +11806,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BH2" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ2" t="n">
+        <v>2147.1</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>2147.1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -11577,6 +11989,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BH3" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ3" t="n">
+        <v>158.6</v>
+      </c>
+      <c r="BK3" t="n">
+        <v>158.6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -11714,6 +12137,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BH4" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ4" t="n">
+        <v>380.7</v>
+      </c>
+      <c r="BK4" t="n">
+        <v>380.7</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -11899,6 +12333,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BH5" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ5" t="n">
+        <v>412</v>
+      </c>
+      <c r="BK5" t="n">
+        <v>412</v>
       </c>
     </row>
     <row r="6">
@@ -12077,6 +12522,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BH6" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ6" t="n">
+        <v>1580</v>
+      </c>
+      <c r="BK6" t="n">
+        <v>1580</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -12252,6 +12708,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BH7" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ7" t="n">
+        <v>1735</v>
+      </c>
+      <c r="BK7" t="n">
+        <v>1735</v>
       </c>
     </row>
     <row r="8">
@@ -12457,6 +12924,22 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BH8" t="inlineStr">
+        <is>
+          <t>enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI8" t="inlineStr">
+        <is>
+          <t>air,enemies,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ8" t="n">
+        <v>4322.2</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>4823.5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12629,6 +13112,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BH9" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ9" t="n">
+        <v>158.2</v>
+      </c>
+      <c r="BK9" t="n">
+        <v>158.2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12806,6 +13300,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BH10" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ10" t="n">
+        <v>521.9</v>
+      </c>
+      <c r="BK10" t="n">
+        <v>521.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -12980,6 +13485,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BH11" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ11" t="n">
+        <v>1733.5</v>
+      </c>
+      <c r="BK11" t="n">
+        <v>1733.5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -13153,6 +13669,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BH12" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ12" t="n">
+        <v>7063</v>
+      </c>
+      <c r="BK12" t="n">
+        <v>7063</v>
       </c>
     </row>
     <row r="13">
@@ -13336,6 +13863,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BH13" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ13" t="n">
+        <v>600</v>
+      </c>
+      <c r="BK13" t="n">
+        <v>600</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -13508,6 +14046,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BH14" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ14" t="n">
+        <v>2677.3</v>
+      </c>
+      <c r="BK14" t="n">
+        <v>2677.3</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -13685,6 +14234,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BH15" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ15" t="n">
+        <v>324</v>
+      </c>
+      <c r="BK15" t="n">
+        <v>324</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -13862,6 +14422,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BH16" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ16" t="n">
+        <v>1247.9</v>
+      </c>
+      <c r="BK16" t="n">
+        <v>1247.9</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -14030,6 +14601,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BH17" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ17" t="n">
+        <v>1193.5</v>
+      </c>
+      <c r="BK17" t="n">
+        <v>1193.5</v>
       </c>
     </row>
     <row r="18">
@@ -14198,6 +14780,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BH18" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ18" t="n">
+        <v>4068.7</v>
+      </c>
+      <c r="BK18" t="n">
+        <v>4068.7</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -14362,6 +14955,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BH19" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ19" t="n">
+        <v>4268.8</v>
+      </c>
+      <c r="BK19" t="n">
+        <v>4268.8</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -14529,6 +15133,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BH20" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ20" t="n">
+        <v>5005.6</v>
+      </c>
+      <c r="BK20" t="n">
+        <v>5005.6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -14706,6 +15321,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BH21" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ21" t="n">
+        <v>4910</v>
+      </c>
+      <c r="BK21" t="n">
+        <v>4910</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -14905,6 +15531,22 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BH22" t="inlineStr">
+        <is>
+          <t>enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI22" t="inlineStr">
+        <is>
+          <t>air,enemies,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ22" t="n">
+        <v>3333.3</v>
+      </c>
+      <c r="BK22" t="n">
+        <v>3333.3</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -14960,7 +15602,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BG23"/>
+  <autoFilter ref="A1:BK23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14971,7 +15613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ21"/>
+  <dimension ref="A1:BD21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -15026,6 +15668,10 @@
     <col width="10" customWidth="1" min="50" max="50"/>
     <col width="13" customWidth="1" min="51" max="51"/>
     <col width="31" customWidth="1" min="52" max="52"/>
+    <col width="31" customWidth="1" min="53" max="53"/>
+    <col width="14" customWidth="1" min="54" max="54"/>
+    <col width="15" customWidth="1" min="55" max="55"/>
+    <col width="12" customWidth="1" min="56" max="56"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -15289,6 +15935,26 @@
           <t>targets_all</t>
         </is>
       </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>atk1_targets</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>atk2_targets</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>dps_vs_ground</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>dps_vs_air</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -15446,6 +16112,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC2" t="n">
+        <v>349.8</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>349.8</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -15604,6 +16281,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BA3" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC3" t="n">
+        <v>107.3</v>
+      </c>
+      <c r="BD3" t="n">
+        <v>107.3</v>
       </c>
     </row>
     <row r="4">
@@ -15772,6 +16460,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA4" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC4" t="n">
+        <v>715.9</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>715.9</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -15879,6 +16578,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA5" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC5" t="n">
+        <v>217.5</v>
+      </c>
+      <c r="BD5" t="n">
+        <v>217.5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -16046,6 +16756,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA6" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC6" t="n">
+        <v>206.6</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>206.6</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -16213,6 +16934,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC7" t="n">
+        <v>535.5</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>535.5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -16370,6 +17102,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC8" t="n">
+        <v>152.5</v>
+      </c>
+      <c r="BD8" t="n">
+        <v>152.5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -16532,6 +17275,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC9" t="n">
+        <v>220</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -16699,6 +17453,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA10" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC10" t="n">
+        <v>300</v>
+      </c>
+      <c r="BD10" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -16866,6 +17631,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA11" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC11" t="n">
+        <v>800</v>
+      </c>
+      <c r="BD11" t="n">
+        <v>800</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -16973,6 +17749,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA12" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC12" t="n">
+        <v>29</v>
+      </c>
+      <c r="BD12" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -17135,6 +17922,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA13" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC13" t="n">
+        <v>469.2</v>
+      </c>
+      <c r="BD13" t="n">
+        <v>469.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -17299,6 +18097,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA14" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC14" t="n">
+        <v>317.5</v>
+      </c>
+      <c r="BD14" t="n">
+        <v>317.5</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -17463,6 +18272,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA15" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC15" t="n">
+        <v>811.2</v>
+      </c>
+      <c r="BD15" t="n">
+        <v>811.2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -17630,6 +18450,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA16" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC16" t="n">
+        <v>470</v>
+      </c>
+      <c r="BD16" t="n">
+        <v>470</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -17797,6 +18628,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA17" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC17" t="n">
+        <v>429</v>
+      </c>
+      <c r="BD17" t="n">
+        <v>429</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -17959,6 +18801,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA18" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC18" t="n">
+        <v>963.5</v>
+      </c>
+      <c r="BD18" t="n">
+        <v>963.5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -18118,6 +18971,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA19" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC19" t="n">
+        <v>2418.8</v>
+      </c>
+      <c r="BD19" t="n">
+        <v>2418.8</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -18281,6 +19145,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BA20" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC20" t="n">
+        <v>7327.7</v>
+      </c>
+      <c r="BD20" t="n">
+        <v>7327.7</v>
       </c>
     </row>
     <row r="21">
@@ -18444,9 +19319,20 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BA21" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BC21" t="n">
+        <v>13333.3</v>
+      </c>
+      <c r="BD21" t="n">
+        <v>13333.3</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AZ21"/>
+  <autoFilter ref="A1:BD21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18457,7 +19343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE22"/>
+  <dimension ref="A1:BI22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -18517,6 +19403,10 @@
     <col width="10" customWidth="1" min="55" max="55"/>
     <col width="13" customWidth="1" min="56" max="56"/>
     <col width="31" customWidth="1" min="57" max="57"/>
+    <col width="31" customWidth="1" min="58" max="58"/>
+    <col width="24" customWidth="1" min="59" max="59"/>
+    <col width="15" customWidth="1" min="60" max="60"/>
+    <col width="12" customWidth="1" min="61" max="61"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -18805,6 +19695,26 @@
           <t>targets_all</t>
         </is>
       </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>atk1_targets</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>atk2_targets</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>dps_vs_ground</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>dps_vs_air</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -18982,6 +19892,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF2" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH2" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>56.9</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -19159,6 +20080,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF3" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH3" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="BI3" t="n">
+        <v>105.5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -19333,6 +20265,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF4" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH4" t="n">
+        <v>246.7</v>
+      </c>
+      <c r="BI4" t="n">
+        <v>246.7</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -19517,6 +20460,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF5" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH5" t="n">
+        <v>477.8</v>
+      </c>
+      <c r="BI5" t="n">
+        <v>477.8</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -19688,6 +20642,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF6" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH6" t="n">
+        <v>781.3</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>781.3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -19858,6 +20823,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BF7" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH7" t="n">
+        <v>1243.1</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>1243.1</v>
       </c>
     </row>
     <row r="8">
@@ -20023,6 +20999,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF8" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH8" t="n">
+        <v>1506.1</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>1506.1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -20190,6 +21177,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF9" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH9" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>176.6</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -20367,6 +21365,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF10" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH10" t="n">
+        <v>318.8</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>318.8</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -20544,6 +21553,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF11" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH11" t="n">
+        <v>1925</v>
+      </c>
+      <c r="BI11" t="n">
+        <v>1925</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -20716,6 +21736,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF12" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH12" t="n">
+        <v>1417.5</v>
+      </c>
+      <c r="BI12" t="n">
+        <v>1417.5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -20891,6 +21922,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BF13" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH13" t="n">
+        <v>2230</v>
+      </c>
+      <c r="BI13" t="n">
+        <v>2230</v>
       </c>
     </row>
     <row r="14">
@@ -21078,6 +22120,19 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF14" t="inlineStr">
+        <is>
+          <t>enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BG14" t="inlineStr">
+        <is>
+          <t>air,enemies,nonancient</t>
+        </is>
+      </c>
+      <c r="BH14" t="n">
+        <v>1998.7</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -21255,6 +22310,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF15" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH15" t="n">
+        <v>641.9</v>
+      </c>
+      <c r="BI15" t="n">
+        <v>641.9</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -21432,6 +22498,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF16" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH16" t="n">
+        <v>2257</v>
+      </c>
+      <c r="BI16" t="n">
+        <v>2257</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -21609,6 +22686,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF17" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH17" t="n">
+        <v>1059.2</v>
+      </c>
+      <c r="BI17" t="n">
+        <v>1059.2</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -21781,6 +22869,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF18" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH18" t="n">
+        <v>1802.5</v>
+      </c>
+      <c r="BI18" t="n">
+        <v>1802.5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -21958,6 +23057,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF19" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH19" t="n">
+        <v>3975.8</v>
+      </c>
+      <c r="BI19" t="n">
+        <v>3975.8</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -22125,6 +23235,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF20" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH20" t="n">
+        <v>7035.7</v>
+      </c>
+      <c r="BI20" t="n">
+        <v>7035.7</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -22344,9 +23465,20 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BF22" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH22" t="n">
+        <v>210.1</v>
+      </c>
+      <c r="BI22" t="n">
+        <v>210.1</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BE22"/>
+  <autoFilter ref="A1:BI22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -22357,7 +23489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BF21"/>
+  <dimension ref="A1:BJ21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -22418,6 +23550,10 @@
     <col width="10" customWidth="1" min="56" max="56"/>
     <col width="13" customWidth="1" min="57" max="57"/>
     <col width="31" customWidth="1" min="58" max="58"/>
+    <col width="31" customWidth="1" min="59" max="59"/>
+    <col width="27" customWidth="1" min="60" max="60"/>
+    <col width="15" customWidth="1" min="61" max="61"/>
+    <col width="12" customWidth="1" min="62" max="62"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -22711,6 +23847,26 @@
           <t>targets_all</t>
         </is>
       </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>atk1_targets</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>atk2_targets</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>dps_vs_ground</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>dps_vs_air</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -22888,6 +24044,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BG2" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI2" t="n">
+        <v>81.2</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>81.2</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -23061,6 +24228,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BG3" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI3" t="n">
+        <v>363.2</v>
+      </c>
+      <c r="BJ3" t="n">
+        <v>363.2</v>
       </c>
     </row>
     <row r="4">
@@ -23239,6 +24417,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BG4" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI4" t="n">
+        <v>132</v>
+      </c>
+      <c r="BJ4" t="n">
+        <v>132</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -23416,6 +24605,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BG5" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI5" t="n">
+        <v>525</v>
+      </c>
+      <c r="BJ5" t="n">
+        <v>525</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -23589,6 +24789,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BG6" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI6" t="n">
+        <v>309.6</v>
+      </c>
+      <c r="BJ6" t="n">
+        <v>309.6</v>
       </c>
     </row>
     <row r="7">
@@ -23762,6 +24973,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BG7" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI7" t="n">
+        <v>1562.5</v>
+      </c>
+      <c r="BJ7" t="n">
+        <v>1562.5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -23934,6 +25156,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BG8" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI8" t="n">
+        <v>813</v>
+      </c>
+      <c r="BJ8" t="n">
+        <v>813</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -24106,6 +25339,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BG9" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI9" t="n">
+        <v>265.5</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>265.5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -24283,6 +25527,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BG10" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI10" t="n">
+        <v>253.7</v>
+      </c>
+      <c r="BJ10" t="n">
+        <v>253.7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -24486,6 +25741,22 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BG11" t="inlineStr">
+        <is>
+          <t>enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH11" t="inlineStr">
+        <is>
+          <t>air,enemies,nonancient</t>
+        </is>
+      </c>
+      <c r="BI11" t="n">
+        <v>6254.3</v>
+      </c>
+      <c r="BJ11" t="n">
+        <v>3273.1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -24660,6 +25931,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BG12" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI12" t="n">
+        <v>986</v>
+      </c>
+      <c r="BJ12" t="n">
+        <v>986</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -24833,6 +26115,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BG13" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI13" t="n">
+        <v>1369.3</v>
+      </c>
+      <c r="BJ13" t="n">
+        <v>1369.3</v>
       </c>
     </row>
     <row r="14">
@@ -25006,6 +26299,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BG14" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI14" t="n">
+        <v>1783</v>
+      </c>
+      <c r="BJ14" t="n">
+        <v>1783</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -25181,6 +26485,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BG15" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI15" t="n">
+        <v>839</v>
+      </c>
+      <c r="BJ15" t="n">
+        <v>839</v>
       </c>
     </row>
     <row r="16">
@@ -25294,6 +26609,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BG16" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI16" t="n">
+        <v>316.7</v>
+      </c>
+      <c r="BJ16" t="n">
+        <v>316.7</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -25466,6 +26792,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BG17" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="BJ17" t="n">
+        <v>1000</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -25670,6 +27007,22 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BG18" t="inlineStr">
+        <is>
+          <t>enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BH18" t="inlineStr">
+        <is>
+          <t>air,enemies,nonancient</t>
+        </is>
+      </c>
+      <c r="BI18" t="n">
+        <v>95.09999999999999</v>
+      </c>
+      <c r="BJ18" t="n">
+        <v>2000</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -25839,6 +27192,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BG19" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI19" t="n">
+        <v>16329.2</v>
+      </c>
+      <c r="BJ19" t="n">
+        <v>16329.2</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -26028,6 +27392,19 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BG20" t="inlineStr">
+        <is>
+          <t>air,enemies,nonancient</t>
+        </is>
+      </c>
+      <c r="BH20" t="inlineStr">
+        <is>
+          <t>enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BJ20" t="n">
+        <v>21721.5</v>
       </c>
     </row>
     <row r="21">
@@ -26190,9 +27567,20 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BG21" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BI21" t="n">
+        <v>897</v>
+      </c>
+      <c r="BJ21" t="n">
+        <v>897</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BF21"/>
+  <autoFilter ref="A1:BJ21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -43875,7 +45263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC20"/>
+  <dimension ref="A1:BG20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -43933,6 +45321,10 @@
     <col width="10" customWidth="1" min="53" max="53"/>
     <col width="13" customWidth="1" min="54" max="54"/>
     <col width="31" customWidth="1" min="55" max="55"/>
+    <col width="31" customWidth="1" min="56" max="56"/>
+    <col width="24" customWidth="1" min="57" max="57"/>
+    <col width="15" customWidth="1" min="58" max="58"/>
+    <col width="12" customWidth="1" min="59" max="59"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -44211,6 +45603,26 @@
           <t>targets_all</t>
         </is>
       </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>atk1_targets</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>atk2_targets</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>dps_vs_ground</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>dps_vs_air</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -44368,6 +45780,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF2" t="n">
+        <v>93.5</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>93.5</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -44525,6 +45948,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BD3" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF3" t="n">
+        <v>779.3</v>
+      </c>
+      <c r="BG3" t="n">
+        <v>779.3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -44684,6 +46118,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BD4" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF4" t="n">
+        <v>218.6</v>
+      </c>
+      <c r="BG4" t="n">
+        <v>218.6</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -44842,6 +46287,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BD5" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF5" t="n">
+        <v>1825.3</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>1825.3</v>
       </c>
     </row>
     <row r="6">
@@ -45005,6 +46461,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BD6" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF6" t="n">
+        <v>175</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>175</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -45172,6 +46639,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BD7" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF7" t="n">
+        <v>2062.6</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>2062.6</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -45325,6 +46803,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BD8" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF8" t="n">
+        <v>3156</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>3156</v>
       </c>
     </row>
     <row r="9">
@@ -45478,6 +46967,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BD9" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF9" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>81.7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -45640,6 +47140,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BD10" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF10" t="n">
+        <v>363</v>
+      </c>
+      <c r="BG10" t="n">
+        <v>363</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -45802,6 +47313,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BD11" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF11" t="n">
+        <v>2007.5</v>
+      </c>
+      <c r="BG11" t="n">
+        <v>2007.5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -45959,6 +47481,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BD12" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF12" t="n">
+        <v>2380</v>
+      </c>
+      <c r="BG12" t="n">
+        <v>2380</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -46114,6 +47647,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BD13" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF13" t="n">
+        <v>9026</v>
+      </c>
+      <c r="BG13" t="n">
+        <v>9026</v>
       </c>
     </row>
     <row r="14">
@@ -46267,6 +47811,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BD14" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF14" t="n">
+        <v>4925.8</v>
+      </c>
+      <c r="BG14" t="n">
+        <v>4925.8</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -46427,6 +47982,17 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BD15" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF15" t="n">
+        <v>727</v>
+      </c>
+      <c r="BG15" t="n">
+        <v>727</v>
       </c>
     </row>
     <row r="16">
@@ -46597,6 +48163,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BD16" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF16" t="n">
+        <v>2118.7</v>
+      </c>
+      <c r="BG16" t="n">
+        <v>2118.7</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -46756,6 +48333,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BD17" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF17" t="n">
+        <v>1807.6</v>
+      </c>
+      <c r="BG17" t="n">
+        <v>1807.6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -46946,6 +48534,22 @@
         <is>
           <t>air,enemies,ground,nonancient</t>
         </is>
+      </c>
+      <c r="BD18" t="inlineStr">
+        <is>
+          <t>enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BE18" t="inlineStr">
+        <is>
+          <t>air,enemies,nonancient</t>
+        </is>
+      </c>
+      <c r="BF18" t="n">
+        <v>1630.5</v>
+      </c>
+      <c r="BG18" t="n">
+        <v>2697.5</v>
       </c>
     </row>
     <row r="19">
@@ -47101,6 +48705,17 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BD19" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF19" t="n">
+        <v>5275</v>
+      </c>
+      <c r="BG19" t="n">
+        <v>5275</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -47258,9 +48873,20 @@
           <t>air,enemies,ground,nonancient</t>
         </is>
       </c>
+      <c r="BD20" t="inlineStr">
+        <is>
+          <t>air,enemies,ground,nonancient</t>
+        </is>
+      </c>
+      <c r="BF20" t="n">
+        <v>8905.6</v>
+      </c>
+      <c r="BG20" t="n">
+        <v>8905.6</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BC20"/>
+  <autoFilter ref="A1:BG20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>